<commit_message>
Update phancong UDM 05
</commit_message>
<xml_diff>
--- a/phancong_UDM_05_dieukhientuxa.xlsx
+++ b/phancong_UDM_05_dieukhientuxa.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\LapTrinhMang\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\GITHUB\UDM_05\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBE8593A-E190-44A4-B149-BD7C78F22788}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88E32CD1-D927-45ED-ADF9-2957B96AC95E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{220251A2-F84B-45B0-B085-A09F5B82D521}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="73">
   <si>
     <t>[UDM_05] - [ Điều khiển và thực thi lệnh từ xa]</t>
   </si>
@@ -99,9 +99,6 @@
     <t>Giới thiệu</t>
   </si>
   <si>
-    <t>Ứng dụng cho phép người dùng kết nối đến một máy Client từ xa sau khi được người dùng tại máy đích cho phép. Khi đã kết nối thành công, người dùng có thể thực thi các lệnh cơ bản nằm trong danh sách cho phép, xem kết quả thực thi, thông báo lỗi và mã kết thúc ngay trên giao diện ứng dụng.</t>
-  </si>
-  <si>
     <t>Kiến trúc hệ thống</t>
   </si>
   <si>
@@ -120,64 +117,10 @@
     <t>Server</t>
   </si>
   <si>
-    <t>Lệnh hoặc các bước chạy Server</t>
-  </si>
-  <si>
-    <t>Lệnh hoặc các bước chạy Client</t>
-  </si>
-  <si>
-    <t>Mô tả cách thay đổi IP, port và các tham số mạng. Không ghi password hoặc secret vào repository.</t>
-  </si>
-  <si>
     <t>Chức năng</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="16"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>Client</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="13"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-  </si>
-  <si>
-    <t>Chức năng 1</t>
-  </si>
-  <si>
-    <t>Chức năng 2</t>
-  </si>
-  <si>
-    <t>Chức năng 3</t>
-  </si>
-  <si>
-    <t>Chức năng 4</t>
-  </si>
-  <si>
-    <t>Chức năng …...</t>
-  </si>
-  <si>
     <t>Kiểm thử</t>
-  </si>
-  <si>
-    <t>Functional test:
-Test dữ liệu không hợp lệ:
-Test mất kết nối:
-Stress test:
-Performance test:
-Bằng chứng kiểm thử lưu tại Extra/.</t>
   </si>
   <si>
     <t>Demo</t>
@@ -191,91 +134,7 @@
     <t>Giới hạn</t>
   </si>
   <si>
-    <t>Liệt kê chức năng chưa hỗ trợ và giới hạn hiện tại của sản phẩm.(Sẽ cập nhật sau khi hoàn thành dự án.)</t>
-  </si>
-  <si>
     <t>Cấu hình</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="16"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">Mô hình: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">Client–Server
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="16"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>Protocol:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> TCP Socket
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="16"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>Port mặc định:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> 5000 (có thể thay đổi)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="16"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>Cấu trúc message:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> Sử dụng mô hình Request/Response, bao gồm các loại message cho yêu cầu kết nối, thực thi lệnh, trả kết quả và yêu cầu dừng lệnh.</t>
-    </r>
   </si>
   <si>
     <r>
@@ -381,11 +240,250 @@
   <si>
     <r>
       <rPr>
+        <b/>
         <sz val="16"/>
         <color theme="1"/>
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
+      <t>Functional Test</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">: Kiểm tra kết nối TCP, thực thi lệnh từ xa, xem danh sách thư mục và ngắt kết nối.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Test dữ liệu không hợp lệ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">: Kiểm tra lệnh không được phép và dữ liệu/request không hợp lệ.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Test kết nối</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">: Kiểm tra xác nhận kết nối, từ chối kết nối và ngắt kết nối.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Stress Test</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">: Kiểm tra Server khi nhiều Client kết nối và gửi yêu cầu đồng thời.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Performance Test</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">: Kiểm tra thời gian phản hồi và khả năng xử lý yêu cầu.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Bằng chứng kiểm thử</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>: Lưu tại thư mục Extra/.</t>
+    </r>
+  </si>
+  <si>
+    <t>Ứng dụng điều khiển và thực thi lệnh từ xa theo mô hình Client–Server. Client kết nối đến Server qua TCP; Server hiển thị yêu cầu và cho phép người dùng tại máy Server chấp nhận hoặc từ chối kết nối. Sau khi được chấp nhận, Client có thể gửi lệnh trong danh sách cho phép, xem kết quả thực thi, xem danh sách thư mục và ngắt kết nối.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Mô hình</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">: Client–Server
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Giao thức</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">: TCP Socket
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Port mặc định</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">: 5000
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Host Server</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">: 0.0.0.0
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Cấu trúc message</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">: Request/Response dạng JSON, gồm action và payload; phản hồi gồm status, output và message.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Xử lý nhiều Client</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>: Server tạo Thread riêng cho từng Client đã được cho phép.</t>
+    </r>
+  </si>
+  <si>
+    <r>
       <t xml:space="preserve">1. Cài đặt môi trường
     Cài đặt Python 3.13.
     Cài đặt Visual Studio Code.
@@ -414,10 +512,177 @@
 3. Kiểm tra Python
     Mở Terminal và chạy:
     python --version
-    Kết quả mong đợi:
+    Kết quả:
     Python 3.13.x 4. Chạy chương trình
-    Chạy Client hoặc Server theo hướng dẫn trong mục Hướng dẫn chạy.</t>
-    </r>
+    Chạy Client và Server theo hướng dẫn trong mục Hướng dẫn chạy.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Client</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Mở một Terminal khác tại thư mục gốc UDM_05 và chạy:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>python Code/Client/client.py</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+Nhập Server IP và Port (mặc định 127.0.0.1 và 5000), sau đó chọn CONNECT. Nếu Server cho phép, Client có thể thực thi lệnh, xem danh sách thư mục và ngắt kết nối.
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Mở Terminal tại thư mục gốc UDM_05 và chạy:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>python Code/Server/server.py</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+Server chạy tại port 5000 và chờ Client kết nối. Khi có Client yêu cầu, Server hiển thị cửa sổ xác nhận để người dùng chọn “Cho phép” hoặc “Từ chối”.
+</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Server sử dụng HOST = 0.0.0.0 và PORT = 5000 trong Code/Server/server.py.
+Client nhập IP và Port Server trực tiếp trên giao diện.
+Khi chạy trên cùng máy: dùng 127.0.0.1:5000.
+Khi chạy qua mạng LAN: nhập địa chỉ IP LAN của máy Server và bảo đảm port 5000 được phép qua tường lửa.
+</t>
+  </si>
+  <si>
+    <t>Kết nối Client–Server qua TCP</t>
+  </si>
+  <si>
+    <t>Xác nhận và từ chối yêu cầu kết nối</t>
+  </si>
+  <si>
+    <t>Xử lý nhiều Client bằng Thread</t>
+  </si>
+  <si>
+    <t>Thực thi lệnh từ xa</t>
+  </si>
+  <si>
+    <t>Kiểm tra và giới hạn lệnh được phép</t>
+  </si>
+  <si>
+    <t>Xem danh sách thư mục</t>
+  </si>
+  <si>
+    <t>Gửi và nhận dữ liệu theo JSON Request/Response</t>
+  </si>
+  <si>
+    <t>Ngắt kết nối Client–Server</t>
+  </si>
+  <si>
+    <t>Xử lý lỗi và mất kết nối</t>
+  </si>
+  <si>
+    <t>Ghi log hoạt động của hệ thống</t>
+  </si>
+  <si>
+    <t>Hệ thống hiện sử dụng TCP Socket và chưa triển khai mã hóa dữ liệu hoặc xác thực tài khoản. Các lệnh thực thi được giới hạn theo whitelist. Một số xử lý lệnh được thiết kế phù hợp với môi trường Windows. Khi triển khai giữa nhiều máy, cần cấu hình đúng địa chỉ IP, port và tường lửa.</t>
+  </si>
+  <si>
+    <t>Danh sách lệnh được phép</t>
+  </si>
+  <si>
+    <t>Hệ thống giới hạn các lệnh thực thi từ xa theo whitelist. Các lệnh được phép gồm:</t>
+  </si>
+  <si>
+    <t>Lệnh</t>
+  </si>
+  <si>
+    <t>ping</t>
+  </si>
+  <si>
+    <t>ipconfig</t>
+  </si>
+  <si>
+    <t>hostname</t>
+  </si>
+  <si>
+    <t>whoami</t>
+  </si>
+  <si>
+    <t>dir</t>
+  </si>
+  <si>
+    <t>echo</t>
+  </si>
+  <si>
+    <t>Các lệnh không nằm trong whitelist sẽ bị từ chối.</t>
+  </si>
+  <si>
+    <t>Hệ thống cũng chặn một số ký tự và toán tử đặc biệt như `;`, `&amp;&amp;`, `||`, `|`, `` ` ``, `$`, `&gt;`, `&lt;` để hạn chế việc thực thi lệnh ngoài phạm vi cho phép.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kiểm tra khả năng kết nối đến địa chỉ mạng </t>
+  </si>
+  <si>
+    <t>Xem thông tin cấu hình mạng</t>
+  </si>
+  <si>
+    <t>Xem tên máy tính</t>
+  </si>
+  <si>
+    <t>Xem tài khoản đang thực thi lệnh</t>
+  </si>
+  <si>
+    <t>Hiển thị nội dung được truyền vào</t>
+  </si>
+  <si>
+    <t>Xem danh sách file và thư mục</t>
   </si>
 </sst>
 </file>
@@ -704,7 +969,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -715,45 +980,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -778,35 +1004,83 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -826,15 +1100,35 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp1.xml><?xml version="1.0" encoding="utf-8"?>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
+</file>
+
+<file path=xl/ctrlProps/ctrlProp10.xml><?xml version="1.0" encoding="utf-8"?>
 <formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
 </file>
 
-<file path=xl/ctrlProps/ctrlProp2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/ctrlProps/ctrlProp11.xml><?xml version="1.0" encoding="utf-8"?>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
+</file>
+
+<file path=xl/ctrlProps/ctrlProp12.xml><?xml version="1.0" encoding="utf-8"?>
 <formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
 </file>
 
+<file path=xl/ctrlProps/ctrlProp13.xml><?xml version="1.0" encoding="utf-8"?>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
+</file>
+
+<file path=xl/ctrlProps/ctrlProp14.xml><?xml version="1.0" encoding="utf-8"?>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
+</file>
+
+<file path=xl/ctrlProps/ctrlProp2.xml><?xml version="1.0" encoding="utf-8"?>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
+</file>
+
 <file path=xl/ctrlProps/ctrlProp3.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp4.xml><?xml version="1.0" encoding="utf-8"?>
@@ -842,7 +1136,23 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp5.xml><?xml version="1.0" encoding="utf-8"?>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
+</file>
+
+<file path=xl/ctrlProps/ctrlProp6.xml><?xml version="1.0" encoding="utf-8"?>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
+</file>
+
+<file path=xl/ctrlProps/ctrlProp7.xml><?xml version="1.0" encoding="utf-8"?>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
+</file>
+
+<file path=xl/ctrlProps/ctrlProp8.xml><?xml version="1.0" encoding="utf-8"?>
 <formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+</file>
+
+<file path=xl/ctrlProps/ctrlProp9.xml><?xml version="1.0" encoding="utf-8"?>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -853,14 +1163,14 @@
         <xdr:from>
           <xdr:col>1</xdr:col>
           <xdr:colOff>579120</xdr:colOff>
-          <xdr:row>44</xdr:row>
+          <xdr:row>59</xdr:row>
           <xdr:rowOff>198120</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>1</xdr:col>
           <xdr:colOff>1211580</xdr:colOff>
-          <xdr:row>45</xdr:row>
-          <xdr:rowOff>240575</xdr:rowOff>
+          <xdr:row>60</xdr:row>
+          <xdr:rowOff>236220</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -920,14 +1230,14 @@
         <xdr:from>
           <xdr:col>1</xdr:col>
           <xdr:colOff>571500</xdr:colOff>
-          <xdr:row>45</xdr:row>
-          <xdr:rowOff>263436</xdr:rowOff>
+          <xdr:row>60</xdr:row>
+          <xdr:rowOff>266700</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>1</xdr:col>
           <xdr:colOff>1203960</xdr:colOff>
-          <xdr:row>46</xdr:row>
-          <xdr:rowOff>243842</xdr:rowOff>
+          <xdr:row>61</xdr:row>
+          <xdr:rowOff>243840</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -987,14 +1297,14 @@
         <xdr:from>
           <xdr:col>1</xdr:col>
           <xdr:colOff>571500</xdr:colOff>
-          <xdr:row>47</xdr:row>
-          <xdr:rowOff>2179</xdr:rowOff>
+          <xdr:row>62</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>1</xdr:col>
           <xdr:colOff>1203960</xdr:colOff>
-          <xdr:row>47</xdr:row>
-          <xdr:rowOff>254727</xdr:rowOff>
+          <xdr:row>62</xdr:row>
+          <xdr:rowOff>251460</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -1054,14 +1364,14 @@
         <xdr:from>
           <xdr:col>1</xdr:col>
           <xdr:colOff>571500</xdr:colOff>
-          <xdr:row>47</xdr:row>
-          <xdr:rowOff>263436</xdr:rowOff>
+          <xdr:row>62</xdr:row>
+          <xdr:rowOff>266700</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>1</xdr:col>
           <xdr:colOff>1203960</xdr:colOff>
-          <xdr:row>48</xdr:row>
-          <xdr:rowOff>243841</xdr:rowOff>
+          <xdr:row>63</xdr:row>
+          <xdr:rowOff>243840</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -1121,14 +1431,14 @@
         <xdr:from>
           <xdr:col>1</xdr:col>
           <xdr:colOff>571500</xdr:colOff>
-          <xdr:row>49</xdr:row>
-          <xdr:rowOff>2179</xdr:rowOff>
+          <xdr:row>69</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>1</xdr:col>
           <xdr:colOff>1203960</xdr:colOff>
-          <xdr:row>49</xdr:row>
-          <xdr:rowOff>254728</xdr:rowOff>
+          <xdr:row>69</xdr:row>
+          <xdr:rowOff>251460</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -1139,6 +1449,609 @@
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
                   <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000009040000}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:extLst>
+              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+                <a14:hiddenFill>
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="65"/>
+                  </a:solidFill>
+                </a14:hiddenFill>
+              </a:ext>
+              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
+                <a14:hiddenLine w="9525">
+                  <a:solidFill>
+                    <a:srgbClr val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
+                  </a:solidFill>
+                  <a:miter lim="800000"/>
+                  <a:headEnd/>
+                  <a:tailEnd/>
+                </a14:hiddenLine>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor editAs="oneCell">
+        <xdr:from>
+          <xdr:col>1</xdr:col>
+          <xdr:colOff>571500</xdr:colOff>
+          <xdr:row>63</xdr:row>
+          <xdr:rowOff>266700</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>1</xdr:col>
+          <xdr:colOff>1203960</xdr:colOff>
+          <xdr:row>64</xdr:row>
+          <xdr:rowOff>243840</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="1056" name="Check Box 32" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s1056"/>
+                </a:ext>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000020040000}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:extLst>
+              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+                <a14:hiddenFill>
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="65"/>
+                  </a:solidFill>
+                </a14:hiddenFill>
+              </a:ext>
+              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
+                <a14:hiddenLine w="9525">
+                  <a:solidFill>
+                    <a:srgbClr val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
+                  </a:solidFill>
+                  <a:miter lim="800000"/>
+                  <a:headEnd/>
+                  <a:tailEnd/>
+                </a14:hiddenLine>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor editAs="oneCell">
+        <xdr:from>
+          <xdr:col>1</xdr:col>
+          <xdr:colOff>571500</xdr:colOff>
+          <xdr:row>64</xdr:row>
+          <xdr:rowOff>266700</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>1</xdr:col>
+          <xdr:colOff>1203960</xdr:colOff>
+          <xdr:row>65</xdr:row>
+          <xdr:rowOff>243840</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="1057" name="Check Box 33" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s1057"/>
+                </a:ext>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000021040000}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:extLst>
+              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+                <a14:hiddenFill>
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="65"/>
+                  </a:solidFill>
+                </a14:hiddenFill>
+              </a:ext>
+              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
+                <a14:hiddenLine w="9525">
+                  <a:solidFill>
+                    <a:srgbClr val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
+                  </a:solidFill>
+                  <a:miter lim="800000"/>
+                  <a:headEnd/>
+                  <a:tailEnd/>
+                </a14:hiddenLine>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor editAs="oneCell">
+        <xdr:from>
+          <xdr:col>1</xdr:col>
+          <xdr:colOff>571500</xdr:colOff>
+          <xdr:row>65</xdr:row>
+          <xdr:rowOff>266700</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>1</xdr:col>
+          <xdr:colOff>1203960</xdr:colOff>
+          <xdr:row>66</xdr:row>
+          <xdr:rowOff>243840</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="1058" name="Check Box 34" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s1058"/>
+                </a:ext>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000022040000}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:extLst>
+              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+                <a14:hiddenFill>
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="65"/>
+                  </a:solidFill>
+                </a14:hiddenFill>
+              </a:ext>
+              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
+                <a14:hiddenLine w="9525">
+                  <a:solidFill>
+                    <a:srgbClr val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
+                  </a:solidFill>
+                  <a:miter lim="800000"/>
+                  <a:headEnd/>
+                  <a:tailEnd/>
+                </a14:hiddenLine>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor editAs="oneCell">
+        <xdr:from>
+          <xdr:col>1</xdr:col>
+          <xdr:colOff>571500</xdr:colOff>
+          <xdr:row>65</xdr:row>
+          <xdr:rowOff>266700</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>1</xdr:col>
+          <xdr:colOff>1203960</xdr:colOff>
+          <xdr:row>66</xdr:row>
+          <xdr:rowOff>243840</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="1059" name="Check Box 35" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s1059"/>
+                </a:ext>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000023040000}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:extLst>
+              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+                <a14:hiddenFill>
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="65"/>
+                  </a:solidFill>
+                </a14:hiddenFill>
+              </a:ext>
+              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
+                <a14:hiddenLine w="9525">
+                  <a:solidFill>
+                    <a:srgbClr val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
+                  </a:solidFill>
+                  <a:miter lim="800000"/>
+                  <a:headEnd/>
+                  <a:tailEnd/>
+                </a14:hiddenLine>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor editAs="oneCell">
+        <xdr:from>
+          <xdr:col>1</xdr:col>
+          <xdr:colOff>571500</xdr:colOff>
+          <xdr:row>66</xdr:row>
+          <xdr:rowOff>266700</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>1</xdr:col>
+          <xdr:colOff>1203960</xdr:colOff>
+          <xdr:row>67</xdr:row>
+          <xdr:rowOff>243840</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="1060" name="Check Box 36" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s1060"/>
+                </a:ext>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000024040000}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:extLst>
+              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+                <a14:hiddenFill>
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="65"/>
+                  </a:solidFill>
+                </a14:hiddenFill>
+              </a:ext>
+              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
+                <a14:hiddenLine w="9525">
+                  <a:solidFill>
+                    <a:srgbClr val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
+                  </a:solidFill>
+                  <a:miter lim="800000"/>
+                  <a:headEnd/>
+                  <a:tailEnd/>
+                </a14:hiddenLine>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor editAs="oneCell">
+        <xdr:from>
+          <xdr:col>1</xdr:col>
+          <xdr:colOff>571500</xdr:colOff>
+          <xdr:row>66</xdr:row>
+          <xdr:rowOff>266700</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>1</xdr:col>
+          <xdr:colOff>1203960</xdr:colOff>
+          <xdr:row>67</xdr:row>
+          <xdr:rowOff>243840</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="1061" name="Check Box 37" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s1061"/>
+                </a:ext>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000025040000}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:extLst>
+              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+                <a14:hiddenFill>
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="65"/>
+                  </a:solidFill>
+                </a14:hiddenFill>
+              </a:ext>
+              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
+                <a14:hiddenLine w="9525">
+                  <a:solidFill>
+                    <a:srgbClr val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
+                  </a:solidFill>
+                  <a:miter lim="800000"/>
+                  <a:headEnd/>
+                  <a:tailEnd/>
+                </a14:hiddenLine>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor editAs="oneCell">
+        <xdr:from>
+          <xdr:col>1</xdr:col>
+          <xdr:colOff>571500</xdr:colOff>
+          <xdr:row>67</xdr:row>
+          <xdr:rowOff>266700</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>1</xdr:col>
+          <xdr:colOff>1203960</xdr:colOff>
+          <xdr:row>68</xdr:row>
+          <xdr:rowOff>243840</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="1062" name="Check Box 38" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s1062"/>
+                </a:ext>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000026040000}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:extLst>
+              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+                <a14:hiddenFill>
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="65"/>
+                  </a:solidFill>
+                </a14:hiddenFill>
+              </a:ext>
+              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
+                <a14:hiddenLine w="9525">
+                  <a:solidFill>
+                    <a:srgbClr val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
+                  </a:solidFill>
+                  <a:miter lim="800000"/>
+                  <a:headEnd/>
+                  <a:tailEnd/>
+                </a14:hiddenLine>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor editAs="oneCell">
+        <xdr:from>
+          <xdr:col>1</xdr:col>
+          <xdr:colOff>571500</xdr:colOff>
+          <xdr:row>67</xdr:row>
+          <xdr:rowOff>266700</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>1</xdr:col>
+          <xdr:colOff>1203960</xdr:colOff>
+          <xdr:row>68</xdr:row>
+          <xdr:rowOff>243840</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="1063" name="Check Box 39" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s1063"/>
+                </a:ext>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000027040000}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:extLst>
+              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+                <a14:hiddenFill>
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="65"/>
+                  </a:solidFill>
+                </a14:hiddenFill>
+              </a:ext>
+              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
+                <a14:hiddenLine w="9525">
+                  <a:solidFill>
+                    <a:srgbClr val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
+                  </a:solidFill>
+                  <a:miter lim="800000"/>
+                  <a:headEnd/>
+                  <a:tailEnd/>
+                </a14:hiddenLine>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor editAs="oneCell">
+        <xdr:from>
+          <xdr:col>1</xdr:col>
+          <xdr:colOff>571500</xdr:colOff>
+          <xdr:row>68</xdr:row>
+          <xdr:rowOff>266700</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>1</xdr:col>
+          <xdr:colOff>1203960</xdr:colOff>
+          <xdr:row>69</xdr:row>
+          <xdr:rowOff>243840</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="1064" name="Check Box 40" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s1064"/>
+                </a:ext>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000028040000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -1482,47 +2395,47 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{956C2DC3-E9A7-488F-9932-70E8B0DD9916}">
-  <dimension ref="A1:M67"/>
+  <dimension ref="A1:M87"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="18.77734375" customWidth="1"/>
-    <col min="3" max="3" width="25.88671875" customWidth="1"/>
+    <col min="3" max="3" width="39.21875" customWidth="1"/>
     <col min="4" max="4" width="37.77734375" customWidth="1"/>
     <col min="5" max="5" width="33.88671875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="25.8" x14ac:dyDescent="0.3">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
-      <c r="K1" s="16"/>
-      <c r="L1" s="16"/>
-      <c r="M1" s="16"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
+      <c r="I1" s="43"/>
+      <c r="J1" s="43"/>
+      <c r="K1" s="43"/>
+      <c r="L1" s="43"/>
+      <c r="M1" s="43"/>
     </row>
     <row r="2" spans="1:13" ht="24.6" x14ac:dyDescent="0.3">
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
-      <c r="G2" s="9"/>
-      <c r="H2" s="9"/>
-      <c r="I2" s="9"/>
-      <c r="J2" s="9"/>
-      <c r="K2" s="9"/>
-      <c r="L2" s="9"/>
-      <c r="M2" s="9"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
+      <c r="I2" s="30"/>
+      <c r="J2" s="30"/>
+      <c r="K2" s="30"/>
+      <c r="L2" s="30"/>
+      <c r="M2" s="30"/>
     </row>
     <row r="3" spans="1:13" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="1"/>
@@ -1561,16 +2474,16 @@
       <c r="M4" s="1"/>
     </row>
     <row r="5" spans="1:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="B5" s="18">
+      <c r="B5" s="5">
         <v>1</v>
       </c>
-      <c r="C5" s="19" t="s">
+      <c r="C5" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="20" t="s">
+      <c r="D5" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="21" t="s">
+      <c r="E5" s="8" t="s">
         <v>17</v>
       </c>
       <c r="F5" s="1"/>
@@ -1583,16 +2496,16 @@
       <c r="M5" s="1"/>
     </row>
     <row r="6" spans="1:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="B6" s="18">
+      <c r="B6" s="5">
         <v>2</v>
       </c>
-      <c r="C6" s="22" t="s">
+      <c r="C6" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="D6" s="20" t="s">
+      <c r="D6" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="23" t="s">
+      <c r="E6" s="10" t="s">
         <v>18</v>
       </c>
       <c r="F6" s="1"/>
@@ -1605,16 +2518,16 @@
       <c r="M6" s="1"/>
     </row>
     <row r="7" spans="1:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="B7" s="18">
+      <c r="B7" s="5">
         <v>3</v>
       </c>
-      <c r="C7" s="24">
+      <c r="C7" s="11">
         <v>2251120375</v>
       </c>
-      <c r="D7" s="20" t="s">
+      <c r="D7" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="E7" s="23" t="s">
+      <c r="E7" s="10" t="s">
         <v>19</v>
       </c>
       <c r="F7" s="1"/>
@@ -1627,16 +2540,16 @@
       <c r="M7" s="1"/>
     </row>
     <row r="8" spans="1:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="B8" s="18">
+      <c r="B8" s="5">
         <v>4</v>
       </c>
-      <c r="C8" s="19" t="s">
+      <c r="C8" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="20" t="s">
+      <c r="D8" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="23" t="s">
+      <c r="E8" s="10" t="s">
         <v>20</v>
       </c>
       <c r="F8" s="1"/>
@@ -1649,16 +2562,16 @@
       <c r="M8" s="1"/>
     </row>
     <row r="9" spans="1:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="B9" s="18">
+      <c r="B9" s="5">
         <v>5</v>
       </c>
-      <c r="C9" s="19" t="s">
+      <c r="C9" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="D9" s="20" t="s">
+      <c r="D9" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="E9" s="23" t="s">
+      <c r="E9" s="10" t="s">
         <v>21</v>
       </c>
       <c r="F9" s="1"/>
@@ -1671,16 +2584,16 @@
       <c r="M9" s="1"/>
     </row>
     <row r="10" spans="1:13" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B10" s="25">
+      <c r="B10" s="12">
         <v>6</v>
       </c>
-      <c r="C10" s="26" t="s">
+      <c r="C10" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="27" t="s">
+      <c r="D10" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="E10" s="28" t="s">
+      <c r="E10" s="15" t="s">
         <v>22</v>
       </c>
       <c r="F10" s="1"/>
@@ -1707,20 +2620,20 @@
       <c r="M11" s="1"/>
     </row>
     <row r="12" spans="1:13" ht="24.6" x14ac:dyDescent="0.3">
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="C12" s="9"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="9"/>
-      <c r="G12" s="9"/>
-      <c r="H12" s="9"/>
-      <c r="I12" s="9"/>
-      <c r="J12" s="9"/>
-      <c r="K12" s="9"/>
-      <c r="L12" s="9"/>
-      <c r="M12" s="9"/>
+      <c r="C12" s="30"/>
+      <c r="D12" s="30"/>
+      <c r="E12" s="30"/>
+      <c r="F12" s="30"/>
+      <c r="G12" s="30"/>
+      <c r="H12" s="30"/>
+      <c r="I12" s="30"/>
+      <c r="J12" s="30"/>
+      <c r="K12" s="30"/>
+      <c r="L12" s="30"/>
+      <c r="M12" s="30"/>
     </row>
     <row r="13" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
       <c r="B13" s="1"/>
@@ -1736,53 +2649,53 @@
       <c r="L13" s="1"/>
       <c r="M13" s="1"/>
     </row>
-    <row r="14" spans="1:13" ht="50.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="31" t="s">
+    <row r="14" spans="1:13" ht="88.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="24" t="s">
+        <v>38</v>
+      </c>
+      <c r="C14" s="24"/>
+      <c r="D14" s="24"/>
+      <c r="E14" s="24"/>
+      <c r="F14" s="24"/>
+      <c r="G14" s="24"/>
+      <c r="H14" s="24"/>
+      <c r="I14" s="24"/>
+      <c r="J14" s="24"/>
+      <c r="K14" s="24"/>
+      <c r="L14" s="24"/>
+      <c r="M14" s="24"/>
+    </row>
+    <row r="15" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="B15" s="41"/>
+      <c r="C15" s="41"/>
+      <c r="D15" s="41"/>
+      <c r="E15" s="41"/>
+      <c r="F15" s="41"/>
+      <c r="G15" s="41"/>
+      <c r="H15" s="41"/>
+      <c r="I15" s="41"/>
+      <c r="J15" s="41"/>
+      <c r="K15" s="41"/>
+      <c r="L15" s="41"/>
+      <c r="M15" s="41"/>
+    </row>
+    <row r="16" spans="1:13" ht="24.6" x14ac:dyDescent="0.3">
+      <c r="B16" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="C14" s="31"/>
-      <c r="D14" s="31"/>
-      <c r="E14" s="31"/>
-      <c r="F14" s="31"/>
-      <c r="G14" s="31"/>
-      <c r="H14" s="31"/>
-      <c r="I14" s="31"/>
-      <c r="J14" s="31"/>
-      <c r="K14" s="31"/>
-      <c r="L14" s="31"/>
-      <c r="M14" s="31"/>
-    </row>
-    <row r="15" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="B15" s="14"/>
-      <c r="C15" s="14"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="14"/>
-      <c r="F15" s="14"/>
-      <c r="G15" s="14"/>
-      <c r="H15" s="14"/>
-      <c r="I15" s="14"/>
-      <c r="J15" s="14"/>
-      <c r="K15" s="14"/>
-      <c r="L15" s="14"/>
-      <c r="M15" s="14"/>
-    </row>
-    <row r="16" spans="1:13" ht="24.6" x14ac:dyDescent="0.3">
-      <c r="B16" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="C16" s="6"/>
-      <c r="D16" s="6"/>
-      <c r="E16" s="6"/>
-      <c r="F16" s="6"/>
-      <c r="G16" s="6"/>
-      <c r="H16" s="6"/>
-      <c r="I16" s="6"/>
-      <c r="J16" s="6"/>
-      <c r="K16" s="6"/>
-      <c r="L16" s="6"/>
-      <c r="M16" s="6"/>
-    </row>
-    <row r="17" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="C16" s="26"/>
+      <c r="D16" s="26"/>
+      <c r="E16" s="26"/>
+      <c r="F16" s="26"/>
+      <c r="G16" s="26"/>
+      <c r="H16" s="26"/>
+      <c r="I16" s="26"/>
+      <c r="J16" s="26"/>
+      <c r="K16" s="26"/>
+      <c r="L16" s="26"/>
+      <c r="M16" s="26"/>
+    </row>
+    <row r="17" spans="1:13" ht="4.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
       <c r="D17" s="1"/>
@@ -1796,21 +2709,21 @@
       <c r="L17" s="1"/>
       <c r="M17" s="1"/>
     </row>
-    <row r="18" spans="1:13" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="32" t="s">
-        <v>48</v>
-      </c>
-      <c r="C18" s="32"/>
-      <c r="D18" s="32"/>
-      <c r="E18" s="32"/>
-      <c r="F18" s="32"/>
-      <c r="G18" s="32"/>
-      <c r="H18" s="32"/>
-      <c r="I18" s="32"/>
-      <c r="J18" s="32"/>
-      <c r="K18" s="32"/>
-      <c r="L18" s="32"/>
-      <c r="M18" s="32"/>
+    <row r="18" spans="1:13" ht="152.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="27" t="s">
+        <v>39</v>
+      </c>
+      <c r="C18" s="27"/>
+      <c r="D18" s="27"/>
+      <c r="E18" s="27"/>
+      <c r="F18" s="27"/>
+      <c r="G18" s="27"/>
+      <c r="H18" s="27"/>
+      <c r="I18" s="27"/>
+      <c r="J18" s="27"/>
+      <c r="K18" s="27"/>
+      <c r="L18" s="27"/>
+      <c r="M18" s="27"/>
     </row>
     <row r="19" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
       <c r="B19" s="1"/>
@@ -1827,20 +2740,20 @@
       <c r="M19" s="1"/>
     </row>
     <row r="20" spans="1:13" ht="24.6" x14ac:dyDescent="0.3">
-      <c r="B20" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="C20" s="9"/>
-      <c r="D20" s="9"/>
-      <c r="E20" s="9"/>
-      <c r="F20" s="9"/>
-      <c r="G20" s="9"/>
-      <c r="H20" s="9"/>
-      <c r="I20" s="9"/>
-      <c r="J20" s="9"/>
-      <c r="K20" s="9"/>
-      <c r="L20" s="9"/>
-      <c r="M20" s="9"/>
+      <c r="B20" s="25" t="s">
+        <v>25</v>
+      </c>
+      <c r="C20" s="30"/>
+      <c r="D20" s="30"/>
+      <c r="E20" s="30"/>
+      <c r="F20" s="30"/>
+      <c r="G20" s="30"/>
+      <c r="H20" s="30"/>
+      <c r="I20" s="30"/>
+      <c r="J20" s="30"/>
+      <c r="K20" s="30"/>
+      <c r="L20" s="30"/>
+      <c r="M20" s="30"/>
     </row>
     <row r="21" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
       <c r="B21" s="1"/>
@@ -1857,20 +2770,20 @@
       <c r="M21" s="1"/>
     </row>
     <row r="22" spans="1:13" ht="124.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="32" t="s">
-        <v>49</v>
-      </c>
-      <c r="C22" s="33"/>
-      <c r="D22" s="33"/>
-      <c r="E22" s="33"/>
-      <c r="F22" s="33"/>
-      <c r="G22" s="33"/>
-      <c r="H22" s="33"/>
-      <c r="I22" s="33"/>
-      <c r="J22" s="33"/>
-      <c r="K22" s="33"/>
-      <c r="L22" s="33"/>
-      <c r="M22" s="33"/>
+      <c r="B22" s="27" t="s">
+        <v>36</v>
+      </c>
+      <c r="C22" s="32"/>
+      <c r="D22" s="32"/>
+      <c r="E22" s="32"/>
+      <c r="F22" s="32"/>
+      <c r="G22" s="32"/>
+      <c r="H22" s="32"/>
+      <c r="I22" s="32"/>
+      <c r="J22" s="32"/>
+      <c r="K22" s="32"/>
+      <c r="L22" s="32"/>
+      <c r="M22" s="32"/>
     </row>
     <row r="23" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
       <c r="B23" s="1"/>
@@ -1887,20 +2800,20 @@
       <c r="M23" s="1"/>
     </row>
     <row r="24" spans="1:13" ht="24.6" x14ac:dyDescent="0.3">
-      <c r="B24" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="C24" s="9"/>
-      <c r="D24" s="9"/>
-      <c r="E24" s="9"/>
-      <c r="F24" s="9"/>
-      <c r="G24" s="9"/>
-      <c r="H24" s="9"/>
-      <c r="I24" s="9"/>
-      <c r="J24" s="9"/>
-      <c r="K24" s="9"/>
-      <c r="L24" s="9"/>
-      <c r="M24" s="9"/>
+      <c r="B24" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="C24" s="30"/>
+      <c r="D24" s="30"/>
+      <c r="E24" s="30"/>
+      <c r="F24" s="30"/>
+      <c r="G24" s="30"/>
+      <c r="H24" s="30"/>
+      <c r="I24" s="30"/>
+      <c r="J24" s="30"/>
+      <c r="K24" s="30"/>
+      <c r="L24" s="30"/>
+      <c r="M24" s="30"/>
     </row>
     <row r="25" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
       <c r="B25" s="1"/>
@@ -1918,20 +2831,20 @@
     </row>
     <row r="26" spans="1:13" ht="281.39999999999998" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
-      <c r="B26" s="34" t="s">
-        <v>50</v>
-      </c>
-      <c r="C26" s="17"/>
-      <c r="D26" s="17"/>
-      <c r="E26" s="17"/>
-      <c r="F26" s="17"/>
-      <c r="G26" s="17"/>
-      <c r="H26" s="17"/>
-      <c r="I26" s="17"/>
-      <c r="J26" s="17"/>
-      <c r="K26" s="17"/>
-      <c r="L26" s="17"/>
-      <c r="M26" s="17"/>
+      <c r="B26" s="31" t="s">
+        <v>40</v>
+      </c>
+      <c r="C26" s="33"/>
+      <c r="D26" s="33"/>
+      <c r="E26" s="33"/>
+      <c r="F26" s="33"/>
+      <c r="G26" s="33"/>
+      <c r="H26" s="33"/>
+      <c r="I26" s="33"/>
+      <c r="J26" s="33"/>
+      <c r="K26" s="33"/>
+      <c r="L26" s="33"/>
+      <c r="M26" s="33"/>
     </row>
     <row r="27" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
@@ -1950,20 +2863,20 @@
     </row>
     <row r="28" spans="1:13" ht="21" x14ac:dyDescent="0.4">
       <c r="A28" s="1"/>
-      <c r="B28" s="35" t="s">
-        <v>28</v>
-      </c>
-      <c r="C28" s="35"/>
-      <c r="D28" s="35"/>
-      <c r="E28" s="35"/>
-      <c r="F28" s="35"/>
-      <c r="G28" s="35"/>
-      <c r="H28" s="35"/>
-      <c r="I28" s="35"/>
-      <c r="J28" s="35"/>
-      <c r="K28" s="35"/>
-      <c r="L28" s="35"/>
-      <c r="M28" s="35"/>
+      <c r="B28" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="C28" s="34"/>
+      <c r="D28" s="34"/>
+      <c r="E28" s="34"/>
+      <c r="F28" s="34"/>
+      <c r="G28" s="34"/>
+      <c r="H28" s="34"/>
+      <c r="I28" s="34"/>
+      <c r="J28" s="34"/>
+      <c r="K28" s="34"/>
+      <c r="L28" s="34"/>
+      <c r="M28" s="34"/>
     </row>
     <row r="29" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
@@ -1982,20 +2895,20 @@
     </row>
     <row r="30" spans="1:13" ht="24.6" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
-      <c r="B30" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="C30" s="6"/>
-      <c r="D30" s="6"/>
-      <c r="E30" s="6"/>
-      <c r="F30" s="6"/>
-      <c r="G30" s="6"/>
-      <c r="H30" s="6"/>
-      <c r="I30" s="6"/>
-      <c r="J30" s="6"/>
-      <c r="K30" s="6"/>
-      <c r="L30" s="6"/>
-      <c r="M30" s="6"/>
+      <c r="B30" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="C30" s="26"/>
+      <c r="D30" s="26"/>
+      <c r="E30" s="26"/>
+      <c r="F30" s="26"/>
+      <c r="G30" s="26"/>
+      <c r="H30" s="26"/>
+      <c r="I30" s="26"/>
+      <c r="J30" s="26"/>
+      <c r="K30" s="26"/>
+      <c r="L30" s="26"/>
+      <c r="M30" s="26"/>
     </row>
     <row r="31" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
@@ -2014,20 +2927,20 @@
     </row>
     <row r="32" spans="1:13" ht="20.399999999999999" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
-      <c r="B32" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="C32" s="11"/>
-      <c r="D32" s="11"/>
-      <c r="E32" s="11"/>
-      <c r="F32" s="11"/>
-      <c r="G32" s="11"/>
-      <c r="H32" s="11"/>
-      <c r="I32" s="11"/>
-      <c r="J32" s="11"/>
-      <c r="K32" s="11"/>
-      <c r="L32" s="11"/>
-      <c r="M32" s="11"/>
+      <c r="B32" s="35" t="s">
+        <v>29</v>
+      </c>
+      <c r="C32" s="36"/>
+      <c r="D32" s="36"/>
+      <c r="E32" s="36"/>
+      <c r="F32" s="36"/>
+      <c r="G32" s="36"/>
+      <c r="H32" s="36"/>
+      <c r="I32" s="36"/>
+      <c r="J32" s="36"/>
+      <c r="K32" s="36"/>
+      <c r="L32" s="36"/>
+      <c r="M32" s="36"/>
     </row>
     <row r="33" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
@@ -2044,22 +2957,22 @@
       <c r="L33" s="1"/>
       <c r="M33" s="1"/>
     </row>
-    <row r="34" spans="1:13" ht="21" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:13" ht="89.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
-      <c r="B34" s="36" t="s">
-        <v>31</v>
-      </c>
-      <c r="C34" s="36"/>
-      <c r="D34" s="36"/>
-      <c r="E34" s="36"/>
-      <c r="F34" s="36"/>
-      <c r="G34" s="36"/>
-      <c r="H34" s="36"/>
-      <c r="I34" s="36"/>
-      <c r="J34" s="36"/>
-      <c r="K34" s="36"/>
-      <c r="L34" s="36"/>
-      <c r="M34" s="36"/>
+      <c r="B34" s="37" t="s">
+        <v>43</v>
+      </c>
+      <c r="C34" s="38"/>
+      <c r="D34" s="38"/>
+      <c r="E34" s="38"/>
+      <c r="F34" s="38"/>
+      <c r="G34" s="38"/>
+      <c r="H34" s="38"/>
+      <c r="I34" s="38"/>
+      <c r="J34" s="38"/>
+      <c r="K34" s="38"/>
+      <c r="L34" s="38"/>
+      <c r="M34" s="38"/>
     </row>
     <row r="35" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
@@ -2078,20 +2991,20 @@
     </row>
     <row r="36" spans="1:13" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
-      <c r="B36" s="12" t="s">
-        <v>35</v>
-      </c>
-      <c r="C36" s="12"/>
-      <c r="D36" s="12"/>
-      <c r="E36" s="12"/>
-      <c r="F36" s="12"/>
-      <c r="G36" s="12"/>
-      <c r="H36" s="12"/>
-      <c r="I36" s="12"/>
-      <c r="J36" s="12"/>
-      <c r="K36" s="12"/>
-      <c r="L36" s="12"/>
-      <c r="M36" s="12"/>
+      <c r="B36" s="31" t="s">
+        <v>41</v>
+      </c>
+      <c r="C36" s="31"/>
+      <c r="D36" s="31"/>
+      <c r="E36" s="31"/>
+      <c r="F36" s="31"/>
+      <c r="G36" s="31"/>
+      <c r="H36" s="31"/>
+      <c r="I36" s="31"/>
+      <c r="J36" s="31"/>
+      <c r="K36" s="31"/>
+      <c r="L36" s="31"/>
+      <c r="M36" s="31"/>
     </row>
     <row r="37" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
@@ -2108,22 +3021,22 @@
       <c r="L37" s="1"/>
       <c r="M37" s="1"/>
     </row>
-    <row r="38" spans="1:13" ht="21" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:13" ht="101.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1"/>
       <c r="B38" s="37" t="s">
-        <v>32</v>
-      </c>
-      <c r="C38" s="37"/>
-      <c r="D38" s="37"/>
-      <c r="E38" s="37"/>
-      <c r="F38" s="37"/>
-      <c r="G38" s="37"/>
-      <c r="H38" s="37"/>
-      <c r="I38" s="37"/>
-      <c r="J38" s="37"/>
-      <c r="K38" s="37"/>
-      <c r="L38" s="37"/>
-      <c r="M38" s="37"/>
+        <v>42</v>
+      </c>
+      <c r="C38" s="38"/>
+      <c r="D38" s="38"/>
+      <c r="E38" s="38"/>
+      <c r="F38" s="38"/>
+      <c r="G38" s="38"/>
+      <c r="H38" s="38"/>
+      <c r="I38" s="38"/>
+      <c r="J38" s="38"/>
+      <c r="K38" s="38"/>
+      <c r="L38" s="38"/>
+      <c r="M38" s="38"/>
     </row>
     <row r="39" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A39" s="1"/>
@@ -2140,22 +3053,22 @@
       <c r="L39" s="1"/>
       <c r="M39" s="1"/>
     </row>
-    <row r="40" spans="1:13" ht="25.2" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:13" ht="20.399999999999999" x14ac:dyDescent="0.35">
       <c r="A40" s="1"/>
-      <c r="B40" s="29" t="s">
-        <v>47</v>
-      </c>
-      <c r="C40" s="13"/>
-      <c r="D40" s="13"/>
-      <c r="E40" s="13"/>
-      <c r="F40" s="13"/>
-      <c r="G40" s="13"/>
-      <c r="H40" s="13"/>
-      <c r="I40" s="13"/>
-      <c r="J40" s="13"/>
-      <c r="K40" s="13"/>
-      <c r="L40" s="13"/>
-      <c r="M40" s="13"/>
+      <c r="B40" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="C40" s="1"/>
+      <c r="D40" s="1"/>
+      <c r="E40" s="1"/>
+      <c r="F40" s="1"/>
+      <c r="G40" s="1"/>
+      <c r="H40" s="1"/>
+      <c r="I40" s="1"/>
+      <c r="J40" s="1"/>
+      <c r="K40" s="1"/>
+      <c r="L40" s="1"/>
+      <c r="M40" s="1"/>
     </row>
     <row r="41" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A41" s="1"/>
@@ -2172,319 +3085,337 @@
       <c r="L41" s="1"/>
       <c r="M41" s="1"/>
     </row>
-    <row r="42" spans="1:13" ht="32.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:13" ht="21" x14ac:dyDescent="0.4">
       <c r="A42" s="1"/>
-      <c r="B42" s="34" t="s">
-        <v>33</v>
-      </c>
-      <c r="C42" s="34"/>
-      <c r="D42" s="34"/>
-      <c r="E42" s="34"/>
-      <c r="F42" s="34"/>
-      <c r="G42" s="34"/>
-      <c r="H42" s="34"/>
-      <c r="I42" s="34"/>
-      <c r="J42" s="34"/>
-      <c r="K42" s="34"/>
-      <c r="L42" s="34"/>
-      <c r="M42" s="34"/>
-    </row>
-    <row r="43" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="B42" s="22" t="s">
+        <v>57</v>
+      </c>
+      <c r="C42" s="22"/>
+      <c r="D42" s="22"/>
+      <c r="E42" s="22"/>
+      <c r="F42" s="22"/>
+      <c r="G42" s="22"/>
+      <c r="H42" s="22"/>
+      <c r="I42" s="22"/>
+      <c r="J42" s="22"/>
+      <c r="K42" s="22"/>
+      <c r="L42" s="22"/>
+      <c r="M42" s="22"/>
+    </row>
+    <row r="43" spans="1:13" ht="21" x14ac:dyDescent="0.4">
       <c r="A43" s="1"/>
-      <c r="B43" s="1"/>
-      <c r="C43" s="1"/>
-      <c r="D43" s="1"/>
-      <c r="E43" s="1"/>
-      <c r="F43" s="1"/>
-      <c r="G43" s="1"/>
-      <c r="H43" s="1"/>
-      <c r="I43" s="1"/>
-      <c r="J43" s="1"/>
-      <c r="K43" s="1"/>
-      <c r="L43" s="1"/>
-      <c r="M43" s="1"/>
-    </row>
-    <row r="44" spans="1:13" ht="24.6" x14ac:dyDescent="0.3">
+      <c r="B43" s="22"/>
+      <c r="C43" s="22"/>
+      <c r="D43" s="22"/>
+      <c r="E43" s="22"/>
+      <c r="F43" s="22"/>
+      <c r="G43" s="22"/>
+      <c r="H43" s="22"/>
+      <c r="I43" s="22"/>
+      <c r="J43" s="22"/>
+      <c r="K43" s="22"/>
+      <c r="L43" s="22"/>
+      <c r="M43" s="22"/>
+    </row>
+    <row r="44" spans="1:13" ht="21" x14ac:dyDescent="0.4">
       <c r="A44" s="1"/>
-      <c r="B44" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="C44" s="5"/>
-      <c r="D44" s="5"/>
-      <c r="E44" s="5"/>
-      <c r="F44" s="5"/>
-      <c r="G44" s="5"/>
-      <c r="H44" s="5"/>
-      <c r="I44" s="5"/>
-      <c r="J44" s="5"/>
-      <c r="K44" s="5"/>
-      <c r="L44" s="5"/>
-      <c r="M44" s="5"/>
-    </row>
-    <row r="45" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="B44" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="C44" s="44" t="s">
+        <v>30</v>
+      </c>
+      <c r="D44" s="44"/>
+      <c r="E44" s="22"/>
+      <c r="F44" s="22"/>
+      <c r="G44" s="22"/>
+      <c r="H44" s="22"/>
+      <c r="I44" s="22"/>
+      <c r="J44" s="22"/>
+      <c r="K44" s="22"/>
+      <c r="L44" s="22"/>
+      <c r="M44" s="22"/>
+    </row>
+    <row r="45" spans="1:13" ht="21" x14ac:dyDescent="0.4">
       <c r="A45" s="1"/>
-      <c r="B45" s="1"/>
-      <c r="C45" s="1"/>
-      <c r="D45" s="1"/>
-      <c r="E45" s="1"/>
-      <c r="F45" s="1"/>
-      <c r="G45" s="1"/>
-      <c r="H45" s="1"/>
-      <c r="I45" s="1"/>
-      <c r="J45" s="1"/>
-      <c r="K45" s="1"/>
-      <c r="L45" s="1"/>
-      <c r="M45" s="1"/>
+      <c r="B45" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="C45" s="45" t="s">
+        <v>67</v>
+      </c>
+      <c r="D45" s="45"/>
+      <c r="E45" s="22"/>
+      <c r="F45" s="22"/>
+      <c r="G45" s="22"/>
+      <c r="H45" s="22"/>
+      <c r="I45" s="22"/>
+      <c r="J45" s="22"/>
+      <c r="K45" s="22"/>
+      <c r="L45" s="22"/>
+      <c r="M45" s="22"/>
     </row>
     <row r="46" spans="1:13" ht="21" x14ac:dyDescent="0.4">
       <c r="A46" s="1"/>
-      <c r="B46" s="30"/>
-      <c r="C46" s="38" t="s">
-        <v>36</v>
-      </c>
-      <c r="D46" s="1"/>
-      <c r="E46" s="1"/>
-      <c r="F46" s="1"/>
-      <c r="G46" s="1"/>
-      <c r="H46" s="1"/>
-      <c r="I46" s="1"/>
-      <c r="J46" s="1"/>
-      <c r="K46" s="1"/>
-      <c r="L46" s="1"/>
-      <c r="M46" s="1"/>
+      <c r="B46" s="23" t="s">
+        <v>60</v>
+      </c>
+      <c r="C46" s="45" t="s">
+        <v>68</v>
+      </c>
+      <c r="D46" s="45"/>
+      <c r="E46" s="22"/>
+      <c r="F46" s="22"/>
+      <c r="G46" s="22"/>
+      <c r="H46" s="22"/>
+      <c r="I46" s="22"/>
+      <c r="J46" s="22"/>
+      <c r="K46" s="22"/>
+      <c r="L46" s="22"/>
+      <c r="M46" s="22"/>
     </row>
     <row r="47" spans="1:13" ht="21" x14ac:dyDescent="0.4">
       <c r="A47" s="1"/>
-      <c r="B47" s="30"/>
-      <c r="C47" s="39" t="s">
-        <v>37</v>
-      </c>
-      <c r="D47" s="1"/>
-      <c r="E47" s="1"/>
-      <c r="F47" s="1"/>
-      <c r="G47" s="1"/>
-      <c r="H47" s="1"/>
-      <c r="I47" s="1"/>
-      <c r="J47" s="1"/>
-      <c r="K47" s="1"/>
-      <c r="L47" s="1"/>
-      <c r="M47" s="1"/>
+      <c r="B47" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="C47" s="45" t="s">
+        <v>69</v>
+      </c>
+      <c r="D47" s="45"/>
+      <c r="E47" s="22"/>
+      <c r="F47" s="22"/>
+      <c r="G47" s="22"/>
+      <c r="H47" s="22"/>
+      <c r="I47" s="22"/>
+      <c r="J47" s="22"/>
+      <c r="K47" s="22"/>
+      <c r="L47" s="22"/>
+      <c r="M47" s="22"/>
     </row>
     <row r="48" spans="1:13" ht="21" x14ac:dyDescent="0.4">
       <c r="A48" s="1"/>
-      <c r="B48" s="30"/>
-      <c r="C48" s="39" t="s">
-        <v>38</v>
-      </c>
-      <c r="D48" s="1"/>
-      <c r="E48" s="1"/>
-      <c r="F48" s="1"/>
-      <c r="G48" s="1"/>
-      <c r="H48" s="1"/>
-      <c r="I48" s="1"/>
-      <c r="J48" s="1"/>
-      <c r="K48" s="1"/>
-      <c r="L48" s="1"/>
-      <c r="M48" s="1"/>
+      <c r="B48" s="23" t="s">
+        <v>62</v>
+      </c>
+      <c r="C48" s="45" t="s">
+        <v>70</v>
+      </c>
+      <c r="D48" s="45"/>
+      <c r="E48" s="22"/>
+      <c r="F48" s="22"/>
+      <c r="G48" s="22"/>
+      <c r="H48" s="22"/>
+      <c r="I48" s="22"/>
+      <c r="J48" s="22"/>
+      <c r="K48" s="22"/>
+      <c r="L48" s="22"/>
+      <c r="M48" s="22"/>
     </row>
     <row r="49" spans="1:13" ht="21" x14ac:dyDescent="0.4">
       <c r="A49" s="1"/>
-      <c r="B49" s="30"/>
-      <c r="C49" s="39" t="s">
-        <v>39</v>
-      </c>
-      <c r="D49" s="1"/>
-      <c r="E49" s="1"/>
-      <c r="F49" s="1"/>
-      <c r="G49" s="1"/>
-      <c r="H49" s="1"/>
-      <c r="I49" s="1"/>
-      <c r="J49" s="1"/>
-      <c r="K49" s="1"/>
-      <c r="L49" s="1"/>
-      <c r="M49" s="1"/>
+      <c r="B49" s="23" t="s">
+        <v>63</v>
+      </c>
+      <c r="C49" s="45" t="s">
+        <v>72</v>
+      </c>
+      <c r="D49" s="45"/>
+      <c r="E49" s="22"/>
+      <c r="F49" s="22"/>
+      <c r="G49" s="22"/>
+      <c r="H49" s="22"/>
+      <c r="I49" s="22"/>
+      <c r="J49" s="22"/>
+      <c r="K49" s="22"/>
+      <c r="L49" s="22"/>
+      <c r="M49" s="22"/>
     </row>
     <row r="50" spans="1:13" ht="21" x14ac:dyDescent="0.4">
       <c r="A50" s="1"/>
-      <c r="B50" s="30"/>
-      <c r="C50" s="39" t="s">
-        <v>40</v>
-      </c>
-      <c r="D50" s="1"/>
-      <c r="E50" s="1"/>
-      <c r="F50" s="1"/>
-      <c r="G50" s="1"/>
-      <c r="H50" s="1"/>
-      <c r="I50" s="1"/>
-      <c r="J50" s="1"/>
-      <c r="K50" s="1"/>
-      <c r="L50" s="1"/>
-      <c r="M50" s="1"/>
-    </row>
-    <row r="51" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="B50" s="23" t="s">
+        <v>64</v>
+      </c>
+      <c r="C50" s="45" t="s">
+        <v>71</v>
+      </c>
+      <c r="D50" s="45"/>
+      <c r="E50" s="22"/>
+      <c r="F50" s="22"/>
+      <c r="G50" s="22"/>
+      <c r="H50" s="22"/>
+      <c r="I50" s="22"/>
+      <c r="J50" s="22"/>
+      <c r="K50" s="22"/>
+      <c r="L50" s="22"/>
+      <c r="M50" s="22"/>
+    </row>
+    <row r="51" spans="1:13" ht="21" x14ac:dyDescent="0.4">
       <c r="A51" s="1"/>
-      <c r="B51" s="1"/>
-      <c r="C51" s="1"/>
-      <c r="D51" s="1"/>
-      <c r="E51" s="1"/>
-      <c r="F51" s="1"/>
-      <c r="G51" s="1"/>
-      <c r="H51" s="1"/>
-      <c r="I51" s="1"/>
-      <c r="J51" s="1"/>
-      <c r="K51" s="1"/>
-      <c r="L51" s="1"/>
-      <c r="M51" s="1"/>
-    </row>
-    <row r="52" spans="1:13" ht="24.6" x14ac:dyDescent="0.3">
+      <c r="B51" s="22"/>
+      <c r="C51" s="22"/>
+      <c r="D51" s="22"/>
+      <c r="E51" s="22"/>
+      <c r="F51" s="22"/>
+      <c r="G51" s="22"/>
+      <c r="H51" s="22"/>
+      <c r="I51" s="22"/>
+      <c r="J51" s="22"/>
+      <c r="K51" s="22"/>
+      <c r="L51" s="22"/>
+      <c r="M51" s="22"/>
+    </row>
+    <row r="52" spans="1:13" ht="21" x14ac:dyDescent="0.4">
       <c r="A52" s="1"/>
-      <c r="B52" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="C52" s="6"/>
-      <c r="D52" s="6"/>
-      <c r="E52" s="6"/>
-      <c r="F52" s="6"/>
-      <c r="G52" s="6"/>
-      <c r="H52" s="6"/>
-      <c r="I52" s="6"/>
-      <c r="J52" s="6"/>
-      <c r="K52" s="6"/>
-      <c r="L52" s="6"/>
-      <c r="M52" s="6"/>
-    </row>
-    <row r="53" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="B52" s="22" t="s">
+        <v>65</v>
+      </c>
+      <c r="C52" s="22"/>
+      <c r="D52" s="22"/>
+      <c r="E52" s="22"/>
+      <c r="F52" s="22"/>
+      <c r="G52" s="22"/>
+      <c r="H52" s="22"/>
+      <c r="I52" s="22"/>
+      <c r="J52" s="22"/>
+      <c r="K52" s="22"/>
+      <c r="L52" s="22"/>
+      <c r="M52" s="22"/>
+    </row>
+    <row r="53" spans="1:13" ht="21" x14ac:dyDescent="0.4">
       <c r="A53" s="1"/>
-      <c r="B53" s="1"/>
-      <c r="C53" s="1"/>
-      <c r="D53" s="1"/>
-      <c r="E53" s="1"/>
-      <c r="F53" s="1"/>
-      <c r="G53" s="1"/>
-      <c r="H53" s="1"/>
-      <c r="I53" s="1"/>
-      <c r="J53" s="1"/>
-      <c r="K53" s="1"/>
-      <c r="L53" s="1"/>
-      <c r="M53" s="1"/>
-    </row>
-    <row r="54" spans="1:13" ht="145.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B53" s="22" t="s">
+        <v>66</v>
+      </c>
+      <c r="C53" s="22"/>
+      <c r="D53" s="22"/>
+      <c r="E53" s="22"/>
+      <c r="F53" s="22"/>
+      <c r="G53" s="22"/>
+      <c r="H53" s="22"/>
+      <c r="I53" s="22"/>
+      <c r="J53" s="22"/>
+      <c r="K53" s="22"/>
+      <c r="L53" s="22"/>
+      <c r="M53" s="22"/>
+    </row>
+    <row r="54" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A54" s="1"/>
-      <c r="B54" s="32" t="s">
-        <v>42</v>
-      </c>
-      <c r="C54" s="32"/>
-      <c r="D54" s="32"/>
-      <c r="E54" s="32"/>
-      <c r="F54" s="32"/>
-      <c r="G54" s="32"/>
-      <c r="H54" s="32"/>
-      <c r="I54" s="32"/>
-      <c r="J54" s="32"/>
-      <c r="K54" s="32"/>
-      <c r="L54" s="32"/>
-      <c r="M54" s="32"/>
-    </row>
-    <row r="55" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="B54" s="1"/>
+      <c r="C54" s="1"/>
+      <c r="D54" s="1"/>
+      <c r="E54" s="1"/>
+      <c r="F54" s="1"/>
+      <c r="G54" s="1"/>
+      <c r="H54" s="1"/>
+      <c r="I54" s="1"/>
+      <c r="J54" s="1"/>
+      <c r="K54" s="1"/>
+      <c r="L54" s="1"/>
+      <c r="M54" s="1"/>
+    </row>
+    <row r="55" spans="1:13" ht="25.2" x14ac:dyDescent="0.3">
       <c r="A55" s="1"/>
-      <c r="B55" s="1"/>
-      <c r="C55" s="1"/>
-      <c r="D55" s="1"/>
-      <c r="E55" s="1"/>
-      <c r="F55" s="1"/>
-      <c r="G55" s="1"/>
-      <c r="H55" s="1"/>
-      <c r="I55" s="1"/>
-      <c r="J55" s="1"/>
-      <c r="K55" s="1"/>
-      <c r="L55" s="1"/>
-      <c r="M55" s="1"/>
-    </row>
-    <row r="56" spans="1:13" ht="25.2" x14ac:dyDescent="0.3">
+      <c r="B55" s="39" t="s">
+        <v>35</v>
+      </c>
+      <c r="C55" s="40"/>
+      <c r="D55" s="40"/>
+      <c r="E55" s="40"/>
+      <c r="F55" s="40"/>
+      <c r="G55" s="40"/>
+      <c r="H55" s="40"/>
+      <c r="I55" s="40"/>
+      <c r="J55" s="40"/>
+      <c r="K55" s="40"/>
+      <c r="L55" s="40"/>
+      <c r="M55" s="40"/>
+    </row>
+    <row r="56" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A56" s="1"/>
-      <c r="B56" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="C56" s="8"/>
-      <c r="D56" s="8"/>
-      <c r="E56" s="8"/>
-      <c r="F56" s="8"/>
-      <c r="G56" s="8"/>
-      <c r="H56" s="8"/>
-      <c r="I56" s="8"/>
-      <c r="J56" s="8"/>
-      <c r="K56" s="8"/>
-      <c r="L56" s="8"/>
-      <c r="M56" s="8"/>
-    </row>
-    <row r="57" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="B56" s="1"/>
+      <c r="C56" s="1"/>
+      <c r="D56" s="1"/>
+      <c r="E56" s="1"/>
+      <c r="F56" s="1"/>
+      <c r="G56" s="1"/>
+      <c r="H56" s="1"/>
+      <c r="I56" s="1"/>
+      <c r="J56" s="1"/>
+      <c r="K56" s="1"/>
+      <c r="L56" s="1"/>
+      <c r="M56" s="1"/>
+    </row>
+    <row r="57" spans="1:13" ht="99.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="1"/>
-      <c r="B57" s="1"/>
-      <c r="C57" s="1"/>
-      <c r="D57" s="1"/>
-      <c r="E57" s="1"/>
-      <c r="F57" s="1"/>
-      <c r="G57" s="1"/>
-      <c r="H57" s="1"/>
-      <c r="I57" s="1"/>
-      <c r="J57" s="1"/>
-      <c r="K57" s="1"/>
-      <c r="L57" s="1"/>
-      <c r="M57" s="1"/>
-    </row>
-    <row r="58" spans="1:13" ht="84" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B57" s="31" t="s">
+        <v>44</v>
+      </c>
+      <c r="C57" s="31"/>
+      <c r="D57" s="31"/>
+      <c r="E57" s="31"/>
+      <c r="F57" s="31"/>
+      <c r="G57" s="31"/>
+      <c r="H57" s="31"/>
+      <c r="I57" s="31"/>
+      <c r="J57" s="31"/>
+      <c r="K57" s="31"/>
+      <c r="L57" s="31"/>
+      <c r="M57" s="31"/>
+    </row>
+    <row r="58" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A58" s="1"/>
-      <c r="B58" s="32" t="s">
-        <v>44</v>
-      </c>
-      <c r="C58" s="32"/>
-      <c r="D58" s="32"/>
-      <c r="E58" s="32"/>
-      <c r="F58" s="32"/>
-      <c r="G58" s="32"/>
-      <c r="H58" s="32"/>
-      <c r="I58" s="32"/>
-      <c r="J58" s="32"/>
-      <c r="K58" s="32"/>
-      <c r="L58" s="32"/>
-      <c r="M58" s="32"/>
-    </row>
-    <row r="59" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="B58" s="1"/>
+      <c r="C58" s="1"/>
+      <c r="D58" s="1"/>
+      <c r="E58" s="1"/>
+      <c r="F58" s="1"/>
+      <c r="G58" s="1"/>
+      <c r="H58" s="1"/>
+      <c r="I58" s="1"/>
+      <c r="J58" s="1"/>
+      <c r="K58" s="1"/>
+      <c r="L58" s="1"/>
+      <c r="M58" s="1"/>
+    </row>
+    <row r="59" spans="1:13" ht="24.6" x14ac:dyDescent="0.3">
       <c r="A59" s="1"/>
-      <c r="B59" s="1"/>
-      <c r="C59" s="1"/>
-      <c r="D59" s="1"/>
-      <c r="E59" s="1"/>
-      <c r="F59" s="1"/>
-      <c r="G59" s="1"/>
-      <c r="H59" s="1"/>
-      <c r="I59" s="1"/>
-      <c r="J59" s="1"/>
-      <c r="K59" s="1"/>
-      <c r="L59" s="1"/>
-      <c r="M59" s="1"/>
-    </row>
-    <row r="60" spans="1:13" ht="24.6" x14ac:dyDescent="0.3">
+      <c r="B59" s="25" t="s">
+        <v>30</v>
+      </c>
+      <c r="C59" s="25"/>
+      <c r="D59" s="25"/>
+      <c r="E59" s="25"/>
+      <c r="F59" s="25"/>
+      <c r="G59" s="25"/>
+      <c r="H59" s="25"/>
+      <c r="I59" s="25"/>
+      <c r="J59" s="25"/>
+      <c r="K59" s="25"/>
+      <c r="L59" s="25"/>
+      <c r="M59" s="25"/>
+    </row>
+    <row r="60" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A60" s="1"/>
-      <c r="B60" s="5" t="s">
+      <c r="B60" s="1"/>
+      <c r="C60" s="1"/>
+      <c r="D60" s="1"/>
+      <c r="E60" s="1"/>
+      <c r="F60" s="1"/>
+      <c r="G60" s="1"/>
+      <c r="H60" s="1"/>
+      <c r="I60" s="1"/>
+      <c r="J60" s="1"/>
+      <c r="K60" s="1"/>
+      <c r="L60" s="1"/>
+      <c r="M60" s="1"/>
+    </row>
+    <row r="61" spans="1:13" ht="21" x14ac:dyDescent="0.4">
+      <c r="A61" s="1"/>
+      <c r="B61" s="16"/>
+      <c r="C61" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="C60" s="9"/>
-      <c r="D60" s="9"/>
-      <c r="E60" s="9"/>
-      <c r="F60" s="9"/>
-      <c r="G60" s="9"/>
-      <c r="H60" s="9"/>
-      <c r="I60" s="9"/>
-      <c r="J60" s="9"/>
-      <c r="K60" s="9"/>
-      <c r="L60" s="9"/>
-      <c r="M60" s="9"/>
-    </row>
-    <row r="61" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A61" s="1"/>
-      <c r="B61" s="1"/>
-      <c r="C61" s="1"/>
       <c r="D61" s="1"/>
       <c r="E61" s="1"/>
       <c r="F61" s="1"/>
@@ -2498,25 +3429,27 @@
     </row>
     <row r="62" spans="1:13" ht="21" x14ac:dyDescent="0.4">
       <c r="A62" s="1"/>
-      <c r="B62" s="40" t="s">
+      <c r="B62" s="16"/>
+      <c r="C62" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="C62" s="40"/>
-      <c r="D62" s="40"/>
-      <c r="E62" s="40"/>
-      <c r="F62" s="40"/>
-      <c r="G62" s="40"/>
-      <c r="H62" s="40"/>
-      <c r="I62" s="40"/>
-      <c r="J62" s="40"/>
-      <c r="K62" s="40"/>
-      <c r="L62" s="40"/>
-      <c r="M62" s="40"/>
-    </row>
-    <row r="63" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="D62" s="1"/>
+      <c r="E62" s="1"/>
+      <c r="F62" s="1"/>
+      <c r="G62" s="1"/>
+      <c r="H62" s="1"/>
+      <c r="I62" s="1"/>
+      <c r="J62" s="1"/>
+      <c r="K62" s="1"/>
+      <c r="L62" s="1"/>
+      <c r="M62" s="1"/>
+    </row>
+    <row r="63" spans="1:13" ht="21" x14ac:dyDescent="0.4">
       <c r="A63" s="1"/>
-      <c r="B63" s="1"/>
-      <c r="C63" s="1"/>
+      <c r="B63" s="16"/>
+      <c r="C63" s="18" t="s">
+        <v>47</v>
+      </c>
       <c r="D63" s="1"/>
       <c r="E63" s="1"/>
       <c r="F63" s="1"/>
@@ -2528,10 +3461,12 @@
       <c r="L63" s="1"/>
       <c r="M63" s="1"/>
     </row>
-    <row r="64" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:13" ht="21" x14ac:dyDescent="0.4">
       <c r="A64" s="1"/>
-      <c r="B64" s="1"/>
-      <c r="C64" s="1"/>
+      <c r="B64" s="16"/>
+      <c r="C64" s="17" t="s">
+        <v>48</v>
+      </c>
       <c r="D64" s="1"/>
       <c r="E64" s="1"/>
       <c r="F64" s="1"/>
@@ -2543,10 +3478,12 @@
       <c r="L64" s="1"/>
       <c r="M64" s="1"/>
     </row>
-    <row r="65" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:13" ht="21" x14ac:dyDescent="0.35">
       <c r="A65" s="1"/>
-      <c r="B65" s="1"/>
-      <c r="C65" s="1"/>
+      <c r="B65" s="16"/>
+      <c r="C65" s="19" t="s">
+        <v>49</v>
+      </c>
       <c r="D65" s="1"/>
       <c r="E65" s="1"/>
       <c r="F65" s="1"/>
@@ -2558,10 +3495,12 @@
       <c r="L65" s="1"/>
       <c r="M65" s="1"/>
     </row>
-    <row r="66" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:13" ht="21" x14ac:dyDescent="0.35">
       <c r="A66" s="1"/>
-      <c r="B66" s="1"/>
-      <c r="C66" s="1"/>
+      <c r="B66" s="16"/>
+      <c r="C66" s="19" t="s">
+        <v>50</v>
+      </c>
       <c r="D66" s="1"/>
       <c r="E66" s="1"/>
       <c r="F66" s="1"/>
@@ -2573,10 +3512,12 @@
       <c r="L66" s="1"/>
       <c r="M66" s="1"/>
     </row>
-    <row r="67" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:13" ht="21" x14ac:dyDescent="0.35">
       <c r="A67" s="1"/>
-      <c r="B67" s="1"/>
-      <c r="C67" s="1"/>
+      <c r="B67" s="16"/>
+      <c r="C67" s="19" t="s">
+        <v>51</v>
+      </c>
       <c r="D67" s="1"/>
       <c r="E67" s="1"/>
       <c r="F67" s="1"/>
@@ -2588,8 +3529,330 @@
       <c r="L67" s="1"/>
       <c r="M67" s="1"/>
     </row>
+    <row r="68" spans="1:13" ht="21" x14ac:dyDescent="0.35">
+      <c r="A68" s="1"/>
+      <c r="B68" s="16"/>
+      <c r="C68" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="D68" s="1"/>
+      <c r="E68" s="1"/>
+      <c r="F68" s="1"/>
+      <c r="G68" s="1"/>
+      <c r="H68" s="1"/>
+      <c r="I68" s="1"/>
+      <c r="J68" s="1"/>
+      <c r="K68" s="1"/>
+      <c r="L68" s="1"/>
+      <c r="M68" s="1"/>
+    </row>
+    <row r="69" spans="1:13" ht="21" x14ac:dyDescent="0.4">
+      <c r="A69" s="1"/>
+      <c r="B69" s="16"/>
+      <c r="C69" s="18" t="s">
+        <v>53</v>
+      </c>
+      <c r="D69" s="1"/>
+      <c r="E69" s="1"/>
+      <c r="F69" s="1"/>
+      <c r="G69" s="1"/>
+      <c r="H69" s="1"/>
+      <c r="I69" s="1"/>
+      <c r="J69" s="1"/>
+      <c r="K69" s="1"/>
+      <c r="L69" s="1"/>
+      <c r="M69" s="1"/>
+    </row>
+    <row r="70" spans="1:13" ht="21" x14ac:dyDescent="0.4">
+      <c r="A70" s="1"/>
+      <c r="B70" s="16"/>
+      <c r="C70" s="18" t="s">
+        <v>54</v>
+      </c>
+      <c r="D70" s="1"/>
+      <c r="E70" s="1"/>
+      <c r="F70" s="1"/>
+      <c r="G70" s="1"/>
+      <c r="H70" s="1"/>
+      <c r="I70" s="1"/>
+      <c r="J70" s="1"/>
+      <c r="K70" s="1"/>
+      <c r="L70" s="1"/>
+      <c r="M70" s="1"/>
+    </row>
+    <row r="71" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A71" s="1"/>
+      <c r="B71" s="1"/>
+      <c r="C71" s="1"/>
+      <c r="D71" s="1"/>
+      <c r="E71" s="1"/>
+      <c r="F71" s="1"/>
+      <c r="G71" s="1"/>
+      <c r="H71" s="1"/>
+      <c r="I71" s="1"/>
+      <c r="J71" s="1"/>
+      <c r="K71" s="1"/>
+      <c r="L71" s="1"/>
+      <c r="M71" s="1"/>
+    </row>
+    <row r="72" spans="1:13" ht="24.6" x14ac:dyDescent="0.3">
+      <c r="A72" s="1"/>
+      <c r="B72" s="25" t="s">
+        <v>31</v>
+      </c>
+      <c r="C72" s="26"/>
+      <c r="D72" s="26"/>
+      <c r="E72" s="26"/>
+      <c r="F72" s="26"/>
+      <c r="G72" s="26"/>
+      <c r="H72" s="26"/>
+      <c r="I72" s="26"/>
+      <c r="J72" s="26"/>
+      <c r="K72" s="26"/>
+      <c r="L72" s="26"/>
+      <c r="M72" s="26"/>
+    </row>
+    <row r="73" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A73" s="1"/>
+      <c r="B73" s="1"/>
+      <c r="C73" s="1"/>
+      <c r="D73" s="1"/>
+      <c r="E73" s="1"/>
+      <c r="F73" s="1"/>
+      <c r="G73" s="1"/>
+      <c r="H73" s="1"/>
+      <c r="I73" s="1"/>
+      <c r="J73" s="1"/>
+      <c r="K73" s="1"/>
+      <c r="L73" s="1"/>
+      <c r="M73" s="1"/>
+    </row>
+    <row r="74" spans="1:13" ht="145.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A74" s="1"/>
+      <c r="B74" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="C74" s="27"/>
+      <c r="D74" s="27"/>
+      <c r="E74" s="27"/>
+      <c r="F74" s="27"/>
+      <c r="G74" s="27"/>
+      <c r="H74" s="27"/>
+      <c r="I74" s="27"/>
+      <c r="J74" s="27"/>
+      <c r="K74" s="27"/>
+      <c r="L74" s="27"/>
+      <c r="M74" s="27"/>
+    </row>
+    <row r="75" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A75" s="1"/>
+      <c r="B75" s="1"/>
+      <c r="C75" s="1"/>
+      <c r="D75" s="1"/>
+      <c r="E75" s="1"/>
+      <c r="F75" s="1"/>
+      <c r="G75" s="1"/>
+      <c r="H75" s="1"/>
+      <c r="I75" s="1"/>
+      <c r="J75" s="1"/>
+      <c r="K75" s="1"/>
+      <c r="L75" s="1"/>
+      <c r="M75" s="1"/>
+    </row>
+    <row r="76" spans="1:13" ht="25.2" x14ac:dyDescent="0.3">
+      <c r="A76" s="1"/>
+      <c r="B76" s="28" t="s">
+        <v>32</v>
+      </c>
+      <c r="C76" s="29"/>
+      <c r="D76" s="29"/>
+      <c r="E76" s="29"/>
+      <c r="F76" s="29"/>
+      <c r="G76" s="29"/>
+      <c r="H76" s="29"/>
+      <c r="I76" s="29"/>
+      <c r="J76" s="29"/>
+      <c r="K76" s="29"/>
+      <c r="L76" s="29"/>
+      <c r="M76" s="29"/>
+    </row>
+    <row r="77" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A77" s="1"/>
+      <c r="B77" s="1"/>
+      <c r="C77" s="1"/>
+      <c r="D77" s="1"/>
+      <c r="E77" s="1"/>
+      <c r="F77" s="1"/>
+      <c r="G77" s="1"/>
+      <c r="H77" s="1"/>
+      <c r="I77" s="1"/>
+      <c r="J77" s="1"/>
+      <c r="K77" s="1"/>
+      <c r="L77" s="1"/>
+      <c r="M77" s="1"/>
+    </row>
+    <row r="78" spans="1:13" ht="84" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A78" s="1"/>
+      <c r="B78" s="27" t="s">
+        <v>33</v>
+      </c>
+      <c r="C78" s="27"/>
+      <c r="D78" s="27"/>
+      <c r="E78" s="27"/>
+      <c r="F78" s="27"/>
+      <c r="G78" s="27"/>
+      <c r="H78" s="27"/>
+      <c r="I78" s="27"/>
+      <c r="J78" s="27"/>
+      <c r="K78" s="27"/>
+      <c r="L78" s="27"/>
+      <c r="M78" s="27"/>
+    </row>
+    <row r="79" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A79" s="1"/>
+      <c r="B79" s="1"/>
+      <c r="C79" s="1"/>
+      <c r="D79" s="1"/>
+      <c r="E79" s="1"/>
+      <c r="F79" s="1"/>
+      <c r="G79" s="1"/>
+      <c r="H79" s="1"/>
+      <c r="I79" s="1"/>
+      <c r="J79" s="1"/>
+      <c r="K79" s="1"/>
+      <c r="L79" s="1"/>
+      <c r="M79" s="1"/>
+    </row>
+    <row r="80" spans="1:13" ht="24.6" x14ac:dyDescent="0.3">
+      <c r="A80" s="1"/>
+      <c r="B80" s="25" t="s">
+        <v>34</v>
+      </c>
+      <c r="C80" s="30"/>
+      <c r="D80" s="30"/>
+      <c r="E80" s="30"/>
+      <c r="F80" s="30"/>
+      <c r="G80" s="30"/>
+      <c r="H80" s="30"/>
+      <c r="I80" s="30"/>
+      <c r="J80" s="30"/>
+      <c r="K80" s="30"/>
+      <c r="L80" s="30"/>
+      <c r="M80" s="30"/>
+    </row>
+    <row r="81" spans="1:13" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A81" s="1"/>
+      <c r="B81" s="1"/>
+      <c r="C81" s="1"/>
+      <c r="D81" s="1"/>
+      <c r="E81" s="1"/>
+      <c r="F81" s="1"/>
+      <c r="G81" s="1"/>
+      <c r="H81" s="1"/>
+      <c r="I81" s="1"/>
+      <c r="J81" s="1"/>
+      <c r="K81" s="1"/>
+      <c r="L81" s="1"/>
+      <c r="M81" s="1"/>
+    </row>
+    <row r="82" spans="1:13" ht="71.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A82" s="1"/>
+      <c r="B82" s="24" t="s">
+        <v>55</v>
+      </c>
+      <c r="C82" s="24"/>
+      <c r="D82" s="24"/>
+      <c r="E82" s="24"/>
+      <c r="F82" s="24"/>
+      <c r="G82" s="24"/>
+      <c r="H82" s="24"/>
+      <c r="I82" s="24"/>
+      <c r="J82" s="24"/>
+      <c r="K82" s="24"/>
+      <c r="L82" s="24"/>
+      <c r="M82" s="24"/>
+    </row>
+    <row r="83" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A83" s="1"/>
+      <c r="B83" s="1"/>
+      <c r="C83" s="1"/>
+      <c r="D83" s="1"/>
+      <c r="E83" s="1"/>
+      <c r="F83" s="1"/>
+      <c r="G83" s="1"/>
+      <c r="H83" s="1"/>
+      <c r="I83" s="1"/>
+      <c r="J83" s="1"/>
+      <c r="K83" s="1"/>
+      <c r="L83" s="1"/>
+      <c r="M83" s="1"/>
+    </row>
+    <row r="84" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A84" s="1"/>
+      <c r="B84" s="1"/>
+      <c r="C84" s="1"/>
+      <c r="D84" s="1"/>
+      <c r="E84" s="1"/>
+      <c r="F84" s="1"/>
+      <c r="G84" s="1"/>
+      <c r="H84" s="1"/>
+      <c r="I84" s="1"/>
+      <c r="J84" s="1"/>
+      <c r="K84" s="1"/>
+      <c r="L84" s="1"/>
+      <c r="M84" s="1"/>
+    </row>
+    <row r="85" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A85" s="1"/>
+      <c r="B85" s="1"/>
+      <c r="C85" s="1"/>
+      <c r="D85" s="1"/>
+      <c r="E85" s="1"/>
+      <c r="F85" s="1"/>
+      <c r="G85" s="1"/>
+      <c r="H85" s="1"/>
+      <c r="I85" s="1"/>
+      <c r="J85" s="1"/>
+      <c r="K85" s="1"/>
+      <c r="L85" s="1"/>
+      <c r="M85" s="1"/>
+    </row>
+    <row r="86" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A86" s="1"/>
+      <c r="B86" s="1"/>
+      <c r="C86" s="1"/>
+      <c r="D86" s="1"/>
+      <c r="E86" s="1"/>
+      <c r="F86" s="1"/>
+      <c r="G86" s="1"/>
+      <c r="H86" s="1"/>
+      <c r="I86" s="1"/>
+      <c r="J86" s="1"/>
+      <c r="K86" s="1"/>
+      <c r="L86" s="1"/>
+      <c r="M86" s="1"/>
+    </row>
+    <row r="87" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A87" s="1"/>
+      <c r="B87" s="1"/>
+      <c r="C87" s="1"/>
+      <c r="D87" s="1"/>
+      <c r="E87" s="1"/>
+      <c r="F87" s="1"/>
+      <c r="G87" s="1"/>
+      <c r="H87" s="1"/>
+      <c r="I87" s="1"/>
+      <c r="J87" s="1"/>
+      <c r="K87" s="1"/>
+      <c r="L87" s="1"/>
+      <c r="M87" s="1"/>
+    </row>
   </sheetData>
-  <mergeCells count="26">
+  <mergeCells count="33">
+    <mergeCell ref="C47:D47"/>
+    <mergeCell ref="C48:D48"/>
+    <mergeCell ref="C49:D49"/>
+    <mergeCell ref="C50:D50"/>
     <mergeCell ref="B14:M14"/>
     <mergeCell ref="B15:M15"/>
     <mergeCell ref="B16:M16"/>
@@ -2597,7 +3860,7 @@
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="B2:M2"/>
     <mergeCell ref="B12:M12"/>
-    <mergeCell ref="B42:M42"/>
+    <mergeCell ref="B57:M57"/>
     <mergeCell ref="B20:M20"/>
     <mergeCell ref="B22:M22"/>
     <mergeCell ref="B24:M24"/>
@@ -2608,14 +3871,17 @@
     <mergeCell ref="B34:M34"/>
     <mergeCell ref="B36:M36"/>
     <mergeCell ref="B38:M38"/>
-    <mergeCell ref="B40:M40"/>
-    <mergeCell ref="B62:M62"/>
-    <mergeCell ref="B44:M44"/>
-    <mergeCell ref="B52:M52"/>
-    <mergeCell ref="B54:M54"/>
-    <mergeCell ref="B56:M56"/>
-    <mergeCell ref="B58:M58"/>
-    <mergeCell ref="B60:M60"/>
+    <mergeCell ref="B55:M55"/>
+    <mergeCell ref="C44:D44"/>
+    <mergeCell ref="C45:D45"/>
+    <mergeCell ref="C46:D46"/>
+    <mergeCell ref="B82:M82"/>
+    <mergeCell ref="B59:M59"/>
+    <mergeCell ref="B72:M72"/>
+    <mergeCell ref="B74:M74"/>
+    <mergeCell ref="B76:M76"/>
+    <mergeCell ref="B78:M78"/>
+    <mergeCell ref="B80:M80"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2631,13 +3897,13 @@
                   <from>
                     <xdr:col>1</xdr:col>
                     <xdr:colOff>579120</xdr:colOff>
-                    <xdr:row>44</xdr:row>
+                    <xdr:row>59</xdr:row>
                     <xdr:rowOff>198120</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>1</xdr:col>
                     <xdr:colOff>1211580</xdr:colOff>
-                    <xdr:row>45</xdr:row>
+                    <xdr:row>60</xdr:row>
                     <xdr:rowOff>236220</xdr:rowOff>
                   </to>
                 </anchor>
@@ -2653,13 +3919,13 @@
                   <from>
                     <xdr:col>1</xdr:col>
                     <xdr:colOff>571500</xdr:colOff>
-                    <xdr:row>45</xdr:row>
+                    <xdr:row>60</xdr:row>
                     <xdr:rowOff>266700</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>1</xdr:col>
                     <xdr:colOff>1203960</xdr:colOff>
-                    <xdr:row>46</xdr:row>
+                    <xdr:row>61</xdr:row>
                     <xdr:rowOff>243840</xdr:rowOff>
                   </to>
                 </anchor>
@@ -2675,13 +3941,13 @@
                   <from>
                     <xdr:col>1</xdr:col>
                     <xdr:colOff>571500</xdr:colOff>
-                    <xdr:row>47</xdr:row>
+                    <xdr:row>62</xdr:row>
                     <xdr:rowOff>0</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>1</xdr:col>
                     <xdr:colOff>1203960</xdr:colOff>
-                    <xdr:row>47</xdr:row>
+                    <xdr:row>62</xdr:row>
                     <xdr:rowOff>251460</xdr:rowOff>
                   </to>
                 </anchor>
@@ -2691,19 +3957,41 @@
         </mc:AlternateContent>
         <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
           <mc:Choice Requires="x14">
-            <control shapeId="1032" r:id="rId6" name="Check Box 8">
+            <control shapeId="1033" r:id="rId6" name="Check Box 9">
               <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
                 <anchor moveWithCells="1">
                   <from>
                     <xdr:col>1</xdr:col>
                     <xdr:colOff>571500</xdr:colOff>
-                    <xdr:row>47</xdr:row>
+                    <xdr:row>69</xdr:row>
+                    <xdr:rowOff>0</xdr:rowOff>
+                  </from>
+                  <to>
+                    <xdr:col>1</xdr:col>
+                    <xdr:colOff>1203960</xdr:colOff>
+                    <xdr:row>69</xdr:row>
+                    <xdr:rowOff>251460</xdr:rowOff>
+                  </to>
+                </anchor>
+              </controlPr>
+            </control>
+          </mc:Choice>
+        </mc:AlternateContent>
+        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+          <mc:Choice Requires="x14">
+            <control shapeId="1032" r:id="rId7" name="Check Box 8">
+              <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
+                <anchor moveWithCells="1">
+                  <from>
+                    <xdr:col>1</xdr:col>
+                    <xdr:colOff>571500</xdr:colOff>
+                    <xdr:row>62</xdr:row>
                     <xdr:rowOff>266700</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>1</xdr:col>
                     <xdr:colOff>1203960</xdr:colOff>
-                    <xdr:row>48</xdr:row>
+                    <xdr:row>63</xdr:row>
                     <xdr:rowOff>243840</xdr:rowOff>
                   </to>
                 </anchor>
@@ -2713,20 +4001,196 @@
         </mc:AlternateContent>
         <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
           <mc:Choice Requires="x14">
-            <control shapeId="1033" r:id="rId7" name="Check Box 9">
+            <control shapeId="1056" r:id="rId8" name="Check Box 32">
               <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
                 <anchor moveWithCells="1">
                   <from>
                     <xdr:col>1</xdr:col>
                     <xdr:colOff>571500</xdr:colOff>
-                    <xdr:row>49</xdr:row>
-                    <xdr:rowOff>0</xdr:rowOff>
+                    <xdr:row>63</xdr:row>
+                    <xdr:rowOff>266700</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>1</xdr:col>
                     <xdr:colOff>1203960</xdr:colOff>
-                    <xdr:row>49</xdr:row>
-                    <xdr:rowOff>251460</xdr:rowOff>
+                    <xdr:row>64</xdr:row>
+                    <xdr:rowOff>243840</xdr:rowOff>
+                  </to>
+                </anchor>
+              </controlPr>
+            </control>
+          </mc:Choice>
+        </mc:AlternateContent>
+        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+          <mc:Choice Requires="x14">
+            <control shapeId="1057" r:id="rId9" name="Check Box 33">
+              <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
+                <anchor moveWithCells="1">
+                  <from>
+                    <xdr:col>1</xdr:col>
+                    <xdr:colOff>571500</xdr:colOff>
+                    <xdr:row>64</xdr:row>
+                    <xdr:rowOff>266700</xdr:rowOff>
+                  </from>
+                  <to>
+                    <xdr:col>1</xdr:col>
+                    <xdr:colOff>1203960</xdr:colOff>
+                    <xdr:row>65</xdr:row>
+                    <xdr:rowOff>243840</xdr:rowOff>
+                  </to>
+                </anchor>
+              </controlPr>
+            </control>
+          </mc:Choice>
+        </mc:AlternateContent>
+        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+          <mc:Choice Requires="x14">
+            <control shapeId="1058" r:id="rId10" name="Check Box 34">
+              <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
+                <anchor moveWithCells="1">
+                  <from>
+                    <xdr:col>1</xdr:col>
+                    <xdr:colOff>571500</xdr:colOff>
+                    <xdr:row>65</xdr:row>
+                    <xdr:rowOff>266700</xdr:rowOff>
+                  </from>
+                  <to>
+                    <xdr:col>1</xdr:col>
+                    <xdr:colOff>1203960</xdr:colOff>
+                    <xdr:row>66</xdr:row>
+                    <xdr:rowOff>243840</xdr:rowOff>
+                  </to>
+                </anchor>
+              </controlPr>
+            </control>
+          </mc:Choice>
+        </mc:AlternateContent>
+        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+          <mc:Choice Requires="x14">
+            <control shapeId="1059" r:id="rId11" name="Check Box 35">
+              <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
+                <anchor moveWithCells="1">
+                  <from>
+                    <xdr:col>1</xdr:col>
+                    <xdr:colOff>571500</xdr:colOff>
+                    <xdr:row>65</xdr:row>
+                    <xdr:rowOff>266700</xdr:rowOff>
+                  </from>
+                  <to>
+                    <xdr:col>1</xdr:col>
+                    <xdr:colOff>1203960</xdr:colOff>
+                    <xdr:row>66</xdr:row>
+                    <xdr:rowOff>243840</xdr:rowOff>
+                  </to>
+                </anchor>
+              </controlPr>
+            </control>
+          </mc:Choice>
+        </mc:AlternateContent>
+        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+          <mc:Choice Requires="x14">
+            <control shapeId="1060" r:id="rId12" name="Check Box 36">
+              <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
+                <anchor moveWithCells="1">
+                  <from>
+                    <xdr:col>1</xdr:col>
+                    <xdr:colOff>571500</xdr:colOff>
+                    <xdr:row>66</xdr:row>
+                    <xdr:rowOff>266700</xdr:rowOff>
+                  </from>
+                  <to>
+                    <xdr:col>1</xdr:col>
+                    <xdr:colOff>1203960</xdr:colOff>
+                    <xdr:row>67</xdr:row>
+                    <xdr:rowOff>243840</xdr:rowOff>
+                  </to>
+                </anchor>
+              </controlPr>
+            </control>
+          </mc:Choice>
+        </mc:AlternateContent>
+        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+          <mc:Choice Requires="x14">
+            <control shapeId="1061" r:id="rId13" name="Check Box 37">
+              <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
+                <anchor moveWithCells="1">
+                  <from>
+                    <xdr:col>1</xdr:col>
+                    <xdr:colOff>571500</xdr:colOff>
+                    <xdr:row>66</xdr:row>
+                    <xdr:rowOff>266700</xdr:rowOff>
+                  </from>
+                  <to>
+                    <xdr:col>1</xdr:col>
+                    <xdr:colOff>1203960</xdr:colOff>
+                    <xdr:row>67</xdr:row>
+                    <xdr:rowOff>243840</xdr:rowOff>
+                  </to>
+                </anchor>
+              </controlPr>
+            </control>
+          </mc:Choice>
+        </mc:AlternateContent>
+        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+          <mc:Choice Requires="x14">
+            <control shapeId="1062" r:id="rId14" name="Check Box 38">
+              <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
+                <anchor moveWithCells="1">
+                  <from>
+                    <xdr:col>1</xdr:col>
+                    <xdr:colOff>571500</xdr:colOff>
+                    <xdr:row>67</xdr:row>
+                    <xdr:rowOff>266700</xdr:rowOff>
+                  </from>
+                  <to>
+                    <xdr:col>1</xdr:col>
+                    <xdr:colOff>1203960</xdr:colOff>
+                    <xdr:row>68</xdr:row>
+                    <xdr:rowOff>243840</xdr:rowOff>
+                  </to>
+                </anchor>
+              </controlPr>
+            </control>
+          </mc:Choice>
+        </mc:AlternateContent>
+        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+          <mc:Choice Requires="x14">
+            <control shapeId="1063" r:id="rId15" name="Check Box 39">
+              <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
+                <anchor moveWithCells="1">
+                  <from>
+                    <xdr:col>1</xdr:col>
+                    <xdr:colOff>571500</xdr:colOff>
+                    <xdr:row>67</xdr:row>
+                    <xdr:rowOff>266700</xdr:rowOff>
+                  </from>
+                  <to>
+                    <xdr:col>1</xdr:col>
+                    <xdr:colOff>1203960</xdr:colOff>
+                    <xdr:row>68</xdr:row>
+                    <xdr:rowOff>243840</xdr:rowOff>
+                  </to>
+                </anchor>
+              </controlPr>
+            </control>
+          </mc:Choice>
+        </mc:AlternateContent>
+        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+          <mc:Choice Requires="x14">
+            <control shapeId="1064" r:id="rId16" name="Check Box 40">
+              <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
+                <anchor moveWithCells="1">
+                  <from>
+                    <xdr:col>1</xdr:col>
+                    <xdr:colOff>571500</xdr:colOff>
+                    <xdr:row>68</xdr:row>
+                    <xdr:rowOff>266700</xdr:rowOff>
+                  </from>
+                  <to>
+                    <xdr:col>1</xdr:col>
+                    <xdr:colOff>1203960</xdr:colOff>
+                    <xdr:row>69</xdr:row>
+                    <xdr:rowOff>243840</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>

</xml_diff>

<commit_message>
Update project assignment file
</commit_message>
<xml_diff>
--- a/phancong_UDM_05_dieukhientuxa.xlsx
+++ b/phancong_UDM_05_dieukhientuxa.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\GITHUB\UDM_05\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71A78B1C-02BE-4068-AC7C-95A922817A65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7201044-B819-4DBD-BD23-F773654D39CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{220251A2-F84B-45B0-B085-A09F5B82D521}"/>
   </bookViews>
@@ -126,11 +126,6 @@
     <t>Demo</t>
   </si>
   <si>
-    <t>Video: [Public hoặc Unlisted URL]
-Slide: PPTX/
-Báo cáo: DOCX/</t>
-  </si>
-  <si>
     <t>Giới hạn</t>
   </si>
   <si>
@@ -677,6 +672,10 @@
   </si>
   <si>
     <t>Xem danh sách file và thư mục</t>
+  </si>
+  <si>
+    <t>Video: [Public hoặc Unlisted URL]
+Báo cáo: DOCX/</t>
   </si>
 </sst>
 </file>
@@ -1005,11 +1004,11 @@
     </xf>
     <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1020,26 +1019,23 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -1071,14 +1067,17 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2119,37 +2118,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="25.8" x14ac:dyDescent="0.3">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
-      <c r="G1" s="32"/>
-      <c r="H1" s="32"/>
-      <c r="I1" s="32"/>
-      <c r="J1" s="32"/>
-      <c r="K1" s="32"/>
-      <c r="L1" s="32"/>
-      <c r="M1" s="32"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
+      <c r="K1" s="30"/>
+      <c r="L1" s="30"/>
+      <c r="M1" s="30"/>
     </row>
     <row r="2" spans="1:13" ht="24.6" x14ac:dyDescent="0.3">
       <c r="B2" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
-      <c r="G2" s="28"/>
-      <c r="H2" s="28"/>
-      <c r="I2" s="28"/>
-      <c r="J2" s="28"/>
-      <c r="K2" s="28"/>
-      <c r="L2" s="28"/>
-      <c r="M2" s="28"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
+      <c r="H2" s="31"/>
+      <c r="I2" s="31"/>
+      <c r="J2" s="31"/>
+      <c r="K2" s="31"/>
+      <c r="L2" s="31"/>
+      <c r="M2" s="31"/>
     </row>
     <row r="3" spans="1:13" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="1"/>
@@ -2337,17 +2336,17 @@
       <c r="B12" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="C12" s="28"/>
-      <c r="D12" s="28"/>
-      <c r="E12" s="28"/>
-      <c r="F12" s="28"/>
-      <c r="G12" s="28"/>
-      <c r="H12" s="28"/>
-      <c r="I12" s="28"/>
-      <c r="J12" s="28"/>
-      <c r="K12" s="28"/>
-      <c r="L12" s="28"/>
-      <c r="M12" s="28"/>
+      <c r="C12" s="31"/>
+      <c r="D12" s="31"/>
+      <c r="E12" s="31"/>
+      <c r="F12" s="31"/>
+      <c r="G12" s="31"/>
+      <c r="H12" s="31"/>
+      <c r="I12" s="31"/>
+      <c r="J12" s="31"/>
+      <c r="K12" s="31"/>
+      <c r="L12" s="31"/>
+      <c r="M12" s="31"/>
     </row>
     <row r="13" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
       <c r="B13" s="1"/>
@@ -2364,34 +2363,34 @@
       <c r="M13" s="1"/>
     </row>
     <row r="14" spans="1:13" ht="88.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="C14" s="22"/>
-      <c r="D14" s="22"/>
-      <c r="E14" s="22"/>
-      <c r="F14" s="22"/>
-      <c r="G14" s="22"/>
-      <c r="H14" s="22"/>
-      <c r="I14" s="22"/>
-      <c r="J14" s="22"/>
-      <c r="K14" s="22"/>
-      <c r="L14" s="22"/>
-      <c r="M14" s="22"/>
+      <c r="B14" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="C14" s="21"/>
+      <c r="D14" s="21"/>
+      <c r="E14" s="21"/>
+      <c r="F14" s="21"/>
+      <c r="G14" s="21"/>
+      <c r="H14" s="21"/>
+      <c r="I14" s="21"/>
+      <c r="J14" s="21"/>
+      <c r="K14" s="21"/>
+      <c r="L14" s="21"/>
+      <c r="M14" s="21"/>
     </row>
     <row r="15" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="B15" s="45"/>
-      <c r="C15" s="45"/>
-      <c r="D15" s="45"/>
-      <c r="E15" s="45"/>
-      <c r="F15" s="45"/>
-      <c r="G15" s="45"/>
-      <c r="H15" s="45"/>
-      <c r="I15" s="45"/>
-      <c r="J15" s="45"/>
-      <c r="K15" s="45"/>
-      <c r="L15" s="45"/>
-      <c r="M15" s="45"/>
+      <c r="B15" s="22"/>
+      <c r="C15" s="22"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="22"/>
+      <c r="F15" s="22"/>
+      <c r="G15" s="22"/>
+      <c r="H15" s="22"/>
+      <c r="I15" s="22"/>
+      <c r="J15" s="22"/>
+      <c r="K15" s="22"/>
+      <c r="L15" s="22"/>
+      <c r="M15" s="22"/>
     </row>
     <row r="16" spans="1:13" ht="24.6" x14ac:dyDescent="0.3">
       <c r="B16" s="23" t="s">
@@ -2425,7 +2424,7 @@
     </row>
     <row r="18" spans="1:13" ht="152.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="25" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C18" s="25"/>
       <c r="D18" s="25"/>
@@ -2457,17 +2456,17 @@
       <c r="B20" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="C20" s="28"/>
-      <c r="D20" s="28"/>
-      <c r="E20" s="28"/>
-      <c r="F20" s="28"/>
-      <c r="G20" s="28"/>
-      <c r="H20" s="28"/>
-      <c r="I20" s="28"/>
-      <c r="J20" s="28"/>
-      <c r="K20" s="28"/>
-      <c r="L20" s="28"/>
-      <c r="M20" s="28"/>
+      <c r="C20" s="31"/>
+      <c r="D20" s="31"/>
+      <c r="E20" s="31"/>
+      <c r="F20" s="31"/>
+      <c r="G20" s="31"/>
+      <c r="H20" s="31"/>
+      <c r="I20" s="31"/>
+      <c r="J20" s="31"/>
+      <c r="K20" s="31"/>
+      <c r="L20" s="31"/>
+      <c r="M20" s="31"/>
     </row>
     <row r="21" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
       <c r="B21" s="1"/>
@@ -2485,19 +2484,19 @@
     </row>
     <row r="22" spans="1:13" ht="124.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22" s="25" t="s">
-        <v>36</v>
-      </c>
-      <c r="C22" s="34"/>
-      <c r="D22" s="34"/>
-      <c r="E22" s="34"/>
-      <c r="F22" s="34"/>
-      <c r="G22" s="34"/>
-      <c r="H22" s="34"/>
-      <c r="I22" s="34"/>
-      <c r="J22" s="34"/>
-      <c r="K22" s="34"/>
-      <c r="L22" s="34"/>
-      <c r="M22" s="34"/>
+        <v>35</v>
+      </c>
+      <c r="C22" s="33"/>
+      <c r="D22" s="33"/>
+      <c r="E22" s="33"/>
+      <c r="F22" s="33"/>
+      <c r="G22" s="33"/>
+      <c r="H22" s="33"/>
+      <c r="I22" s="33"/>
+      <c r="J22" s="33"/>
+      <c r="K22" s="33"/>
+      <c r="L22" s="33"/>
+      <c r="M22" s="33"/>
     </row>
     <row r="23" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
       <c r="B23" s="1"/>
@@ -2517,17 +2516,17 @@
       <c r="B24" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="C24" s="28"/>
-      <c r="D24" s="28"/>
-      <c r="E24" s="28"/>
-      <c r="F24" s="28"/>
-      <c r="G24" s="28"/>
-      <c r="H24" s="28"/>
-      <c r="I24" s="28"/>
-      <c r="J24" s="28"/>
-      <c r="K24" s="28"/>
-      <c r="L24" s="28"/>
-      <c r="M24" s="28"/>
+      <c r="C24" s="31"/>
+      <c r="D24" s="31"/>
+      <c r="E24" s="31"/>
+      <c r="F24" s="31"/>
+      <c r="G24" s="31"/>
+      <c r="H24" s="31"/>
+      <c r="I24" s="31"/>
+      <c r="J24" s="31"/>
+      <c r="K24" s="31"/>
+      <c r="L24" s="31"/>
+      <c r="M24" s="31"/>
     </row>
     <row r="25" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
       <c r="B25" s="1"/>
@@ -2545,20 +2544,20 @@
     </row>
     <row r="26" spans="1:13" ht="281.39999999999998" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
-      <c r="B26" s="33" t="s">
-        <v>40</v>
-      </c>
-      <c r="C26" s="35"/>
-      <c r="D26" s="35"/>
-      <c r="E26" s="35"/>
-      <c r="F26" s="35"/>
-      <c r="G26" s="35"/>
-      <c r="H26" s="35"/>
-      <c r="I26" s="35"/>
-      <c r="J26" s="35"/>
-      <c r="K26" s="35"/>
-      <c r="L26" s="35"/>
-      <c r="M26" s="35"/>
+      <c r="B26" s="32" t="s">
+        <v>39</v>
+      </c>
+      <c r="C26" s="34"/>
+      <c r="D26" s="34"/>
+      <c r="E26" s="34"/>
+      <c r="F26" s="34"/>
+      <c r="G26" s="34"/>
+      <c r="H26" s="34"/>
+      <c r="I26" s="34"/>
+      <c r="J26" s="34"/>
+      <c r="K26" s="34"/>
+      <c r="L26" s="34"/>
+      <c r="M26" s="34"/>
     </row>
     <row r="27" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
@@ -2577,20 +2576,20 @@
     </row>
     <row r="28" spans="1:13" ht="21" x14ac:dyDescent="0.4">
       <c r="A28" s="1"/>
-      <c r="B28" s="36" t="s">
+      <c r="B28" s="35" t="s">
         <v>27</v>
       </c>
-      <c r="C28" s="36"/>
-      <c r="D28" s="36"/>
-      <c r="E28" s="36"/>
-      <c r="F28" s="36"/>
-      <c r="G28" s="36"/>
-      <c r="H28" s="36"/>
-      <c r="I28" s="36"/>
-      <c r="J28" s="36"/>
-      <c r="K28" s="36"/>
-      <c r="L28" s="36"/>
-      <c r="M28" s="36"/>
+      <c r="C28" s="35"/>
+      <c r="D28" s="35"/>
+      <c r="E28" s="35"/>
+      <c r="F28" s="35"/>
+      <c r="G28" s="35"/>
+      <c r="H28" s="35"/>
+      <c r="I28" s="35"/>
+      <c r="J28" s="35"/>
+      <c r="K28" s="35"/>
+      <c r="L28" s="35"/>
+      <c r="M28" s="35"/>
     </row>
     <row r="29" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
@@ -2641,20 +2640,20 @@
     </row>
     <row r="32" spans="1:13" ht="20.399999999999999" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
-      <c r="B32" s="37" t="s">
+      <c r="B32" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="C32" s="38"/>
-      <c r="D32" s="38"/>
-      <c r="E32" s="38"/>
-      <c r="F32" s="38"/>
-      <c r="G32" s="38"/>
-      <c r="H32" s="38"/>
-      <c r="I32" s="38"/>
-      <c r="J32" s="38"/>
-      <c r="K32" s="38"/>
-      <c r="L32" s="38"/>
-      <c r="M32" s="38"/>
+      <c r="C32" s="37"/>
+      <c r="D32" s="37"/>
+      <c r="E32" s="37"/>
+      <c r="F32" s="37"/>
+      <c r="G32" s="37"/>
+      <c r="H32" s="37"/>
+      <c r="I32" s="37"/>
+      <c r="J32" s="37"/>
+      <c r="K32" s="37"/>
+      <c r="L32" s="37"/>
+      <c r="M32" s="37"/>
     </row>
     <row r="33" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
@@ -2673,20 +2672,20 @@
     </row>
     <row r="34" spans="1:13" ht="89.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
-      <c r="B34" s="39" t="s">
-        <v>43</v>
-      </c>
-      <c r="C34" s="40"/>
-      <c r="D34" s="40"/>
-      <c r="E34" s="40"/>
-      <c r="F34" s="40"/>
-      <c r="G34" s="40"/>
-      <c r="H34" s="40"/>
-      <c r="I34" s="40"/>
-      <c r="J34" s="40"/>
-      <c r="K34" s="40"/>
-      <c r="L34" s="40"/>
-      <c r="M34" s="40"/>
+      <c r="B34" s="38" t="s">
+        <v>42</v>
+      </c>
+      <c r="C34" s="39"/>
+      <c r="D34" s="39"/>
+      <c r="E34" s="39"/>
+      <c r="F34" s="39"/>
+      <c r="G34" s="39"/>
+      <c r="H34" s="39"/>
+      <c r="I34" s="39"/>
+      <c r="J34" s="39"/>
+      <c r="K34" s="39"/>
+      <c r="L34" s="39"/>
+      <c r="M34" s="39"/>
     </row>
     <row r="35" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
@@ -2705,20 +2704,20 @@
     </row>
     <row r="36" spans="1:13" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
-      <c r="B36" s="33" t="s">
-        <v>41</v>
-      </c>
-      <c r="C36" s="33"/>
-      <c r="D36" s="33"/>
-      <c r="E36" s="33"/>
-      <c r="F36" s="33"/>
-      <c r="G36" s="33"/>
-      <c r="H36" s="33"/>
-      <c r="I36" s="33"/>
-      <c r="J36" s="33"/>
-      <c r="K36" s="33"/>
-      <c r="L36" s="33"/>
-      <c r="M36" s="33"/>
+      <c r="B36" s="32" t="s">
+        <v>40</v>
+      </c>
+      <c r="C36" s="32"/>
+      <c r="D36" s="32"/>
+      <c r="E36" s="32"/>
+      <c r="F36" s="32"/>
+      <c r="G36" s="32"/>
+      <c r="H36" s="32"/>
+      <c r="I36" s="32"/>
+      <c r="J36" s="32"/>
+      <c r="K36" s="32"/>
+      <c r="L36" s="32"/>
+      <c r="M36" s="32"/>
     </row>
     <row r="37" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
@@ -2737,20 +2736,20 @@
     </row>
     <row r="38" spans="1:13" ht="101.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1"/>
-      <c r="B38" s="39" t="s">
-        <v>42</v>
-      </c>
-      <c r="C38" s="40"/>
-      <c r="D38" s="40"/>
-      <c r="E38" s="40"/>
-      <c r="F38" s="40"/>
-      <c r="G38" s="40"/>
-      <c r="H38" s="40"/>
-      <c r="I38" s="40"/>
-      <c r="J38" s="40"/>
-      <c r="K38" s="40"/>
-      <c r="L38" s="40"/>
-      <c r="M38" s="40"/>
+      <c r="B38" s="38" t="s">
+        <v>41</v>
+      </c>
+      <c r="C38" s="39"/>
+      <c r="D38" s="39"/>
+      <c r="E38" s="39"/>
+      <c r="F38" s="39"/>
+      <c r="G38" s="39"/>
+      <c r="H38" s="39"/>
+      <c r="I38" s="39"/>
+      <c r="J38" s="39"/>
+      <c r="K38" s="39"/>
+      <c r="L38" s="39"/>
+      <c r="M38" s="39"/>
     </row>
     <row r="39" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A39" s="1"/>
@@ -2770,7 +2769,7 @@
     <row r="40" spans="1:13" ht="20.399999999999999" x14ac:dyDescent="0.35">
       <c r="A40" s="1"/>
       <c r="B40" s="17" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C40" s="1"/>
       <c r="D40" s="1"/>
@@ -2802,7 +2801,7 @@
     <row r="42" spans="1:13" ht="21" x14ac:dyDescent="0.4">
       <c r="A42" s="1"/>
       <c r="B42" s="19" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C42" s="19"/>
       <c r="D42" s="19"/>
@@ -2834,12 +2833,12 @@
     <row r="44" spans="1:13" ht="21" x14ac:dyDescent="0.4">
       <c r="A44" s="1"/>
       <c r="B44" s="18" t="s">
-        <v>58</v>
-      </c>
-      <c r="C44" s="43" t="s">
+        <v>57</v>
+      </c>
+      <c r="C44" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="D44" s="43"/>
+      <c r="D44" s="26"/>
       <c r="E44" s="19"/>
       <c r="F44" s="19"/>
       <c r="G44" s="19"/>
@@ -2853,12 +2852,12 @@
     <row r="45" spans="1:13" ht="21" x14ac:dyDescent="0.4">
       <c r="A45" s="1"/>
       <c r="B45" s="20" t="s">
-        <v>59</v>
-      </c>
-      <c r="C45" s="44" t="s">
-        <v>66</v>
-      </c>
-      <c r="D45" s="44"/>
+        <v>58</v>
+      </c>
+      <c r="C45" s="27" t="s">
+        <v>65</v>
+      </c>
+      <c r="D45" s="27"/>
       <c r="E45" s="19"/>
       <c r="F45" s="19"/>
       <c r="G45" s="19"/>
@@ -2872,12 +2871,12 @@
     <row r="46" spans="1:13" ht="21" x14ac:dyDescent="0.4">
       <c r="A46" s="1"/>
       <c r="B46" s="20" t="s">
-        <v>60</v>
-      </c>
-      <c r="C46" s="44" t="s">
-        <v>67</v>
-      </c>
-      <c r="D46" s="44"/>
+        <v>59</v>
+      </c>
+      <c r="C46" s="27" t="s">
+        <v>66</v>
+      </c>
+      <c r="D46" s="27"/>
       <c r="E46" s="19"/>
       <c r="F46" s="19"/>
       <c r="G46" s="19"/>
@@ -2891,12 +2890,12 @@
     <row r="47" spans="1:13" ht="21" x14ac:dyDescent="0.4">
       <c r="A47" s="1"/>
       <c r="B47" s="20" t="s">
-        <v>61</v>
-      </c>
-      <c r="C47" s="44" t="s">
-        <v>68</v>
-      </c>
-      <c r="D47" s="44"/>
+        <v>60</v>
+      </c>
+      <c r="C47" s="27" t="s">
+        <v>67</v>
+      </c>
+      <c r="D47" s="27"/>
       <c r="E47" s="19"/>
       <c r="F47" s="19"/>
       <c r="G47" s="19"/>
@@ -2910,12 +2909,12 @@
     <row r="48" spans="1:13" ht="21" x14ac:dyDescent="0.4">
       <c r="A48" s="1"/>
       <c r="B48" s="20" t="s">
-        <v>62</v>
-      </c>
-      <c r="C48" s="44" t="s">
-        <v>70</v>
-      </c>
-      <c r="D48" s="44"/>
+        <v>61</v>
+      </c>
+      <c r="C48" s="27" t="s">
+        <v>69</v>
+      </c>
+      <c r="D48" s="27"/>
       <c r="E48" s="19"/>
       <c r="F48" s="19"/>
       <c r="G48" s="19"/>
@@ -2929,12 +2928,12 @@
     <row r="49" spans="1:13" ht="21" x14ac:dyDescent="0.4">
       <c r="A49" s="1"/>
       <c r="B49" s="20" t="s">
-        <v>63</v>
-      </c>
-      <c r="C49" s="44" t="s">
-        <v>69</v>
-      </c>
-      <c r="D49" s="44"/>
+        <v>62</v>
+      </c>
+      <c r="C49" s="27" t="s">
+        <v>68</v>
+      </c>
+      <c r="D49" s="27"/>
       <c r="E49" s="19"/>
       <c r="F49" s="19"/>
       <c r="G49" s="19"/>
@@ -2963,7 +2962,7 @@
     <row r="51" spans="1:13" ht="21" x14ac:dyDescent="0.4">
       <c r="A51" s="1"/>
       <c r="B51" s="19" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C51" s="19"/>
       <c r="D51" s="19"/>
@@ -2980,7 +2979,7 @@
     <row r="52" spans="1:13" ht="21" x14ac:dyDescent="0.4">
       <c r="A52" s="1"/>
       <c r="B52" s="19" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C52" s="19"/>
       <c r="D52" s="19"/>
@@ -3011,20 +3010,20 @@
     </row>
     <row r="54" spans="1:13" ht="25.2" x14ac:dyDescent="0.3">
       <c r="A54" s="1"/>
-      <c r="B54" s="41" t="s">
-        <v>35</v>
-      </c>
-      <c r="C54" s="42"/>
-      <c r="D54" s="42"/>
-      <c r="E54" s="42"/>
-      <c r="F54" s="42"/>
-      <c r="G54" s="42"/>
-      <c r="H54" s="42"/>
-      <c r="I54" s="42"/>
-      <c r="J54" s="42"/>
-      <c r="K54" s="42"/>
-      <c r="L54" s="42"/>
-      <c r="M54" s="42"/>
+      <c r="B54" s="40" t="s">
+        <v>34</v>
+      </c>
+      <c r="C54" s="41"/>
+      <c r="D54" s="41"/>
+      <c r="E54" s="41"/>
+      <c r="F54" s="41"/>
+      <c r="G54" s="41"/>
+      <c r="H54" s="41"/>
+      <c r="I54" s="41"/>
+      <c r="J54" s="41"/>
+      <c r="K54" s="41"/>
+      <c r="L54" s="41"/>
+      <c r="M54" s="41"/>
     </row>
     <row r="55" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A55" s="1"/>
@@ -3043,20 +3042,20 @@
     </row>
     <row r="56" spans="1:13" ht="99.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="1"/>
-      <c r="B56" s="33" t="s">
-        <v>44</v>
-      </c>
-      <c r="C56" s="33"/>
-      <c r="D56" s="33"/>
-      <c r="E56" s="33"/>
-      <c r="F56" s="33"/>
-      <c r="G56" s="33"/>
-      <c r="H56" s="33"/>
-      <c r="I56" s="33"/>
-      <c r="J56" s="33"/>
-      <c r="K56" s="33"/>
-      <c r="L56" s="33"/>
-      <c r="M56" s="33"/>
+      <c r="B56" s="32" t="s">
+        <v>43</v>
+      </c>
+      <c r="C56" s="32"/>
+      <c r="D56" s="32"/>
+      <c r="E56" s="32"/>
+      <c r="F56" s="32"/>
+      <c r="G56" s="32"/>
+      <c r="H56" s="32"/>
+      <c r="I56" s="32"/>
+      <c r="J56" s="32"/>
+      <c r="K56" s="32"/>
+      <c r="L56" s="32"/>
+      <c r="M56" s="32"/>
     </row>
     <row r="57" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A57" s="1"/>
@@ -3108,10 +3107,10 @@
     <row r="60" spans="1:13" ht="21" x14ac:dyDescent="0.35">
       <c r="A60" s="1"/>
       <c r="B60" s="16"/>
-      <c r="C60" s="29" t="s">
-        <v>45</v>
-      </c>
-      <c r="D60" s="29"/>
+      <c r="C60" s="44" t="s">
+        <v>44</v>
+      </c>
+      <c r="D60" s="44"/>
       <c r="E60" s="1"/>
       <c r="F60" s="1"/>
       <c r="G60" s="1"/>
@@ -3125,10 +3124,10 @@
     <row r="61" spans="1:13" ht="21" x14ac:dyDescent="0.35">
       <c r="A61" s="1"/>
       <c r="B61" s="16"/>
-      <c r="C61" s="21" t="s">
-        <v>46</v>
-      </c>
-      <c r="D61" s="21"/>
+      <c r="C61" s="28" t="s">
+        <v>45</v>
+      </c>
+      <c r="D61" s="28"/>
       <c r="E61" s="1"/>
       <c r="F61" s="1"/>
       <c r="G61" s="1"/>
@@ -3142,10 +3141,10 @@
     <row r="62" spans="1:13" ht="21" x14ac:dyDescent="0.35">
       <c r="A62" s="1"/>
       <c r="B62" s="16"/>
-      <c r="C62" s="21" t="s">
-        <v>47</v>
-      </c>
-      <c r="D62" s="21"/>
+      <c r="C62" s="28" t="s">
+        <v>46</v>
+      </c>
+      <c r="D62" s="28"/>
       <c r="E62" s="1"/>
       <c r="F62" s="1"/>
       <c r="G62" s="1"/>
@@ -3159,10 +3158,10 @@
     <row r="63" spans="1:13" ht="21" x14ac:dyDescent="0.35">
       <c r="A63" s="1"/>
       <c r="B63" s="16"/>
-      <c r="C63" s="29" t="s">
-        <v>48</v>
-      </c>
-      <c r="D63" s="29"/>
+      <c r="C63" s="44" t="s">
+        <v>47</v>
+      </c>
+      <c r="D63" s="44"/>
       <c r="E63" s="1"/>
       <c r="F63" s="1"/>
       <c r="G63" s="1"/>
@@ -3176,10 +3175,10 @@
     <row r="64" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A64" s="1"/>
       <c r="B64" s="16"/>
-      <c r="C64" s="30" t="s">
-        <v>49</v>
-      </c>
-      <c r="D64" s="30"/>
+      <c r="C64" s="45" t="s">
+        <v>48</v>
+      </c>
+      <c r="D64" s="45"/>
       <c r="E64" s="1"/>
       <c r="F64" s="1"/>
       <c r="G64" s="1"/>
@@ -3193,10 +3192,10 @@
     <row r="65" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A65" s="1"/>
       <c r="B65" s="16"/>
-      <c r="C65" s="30" t="s">
-        <v>50</v>
-      </c>
-      <c r="D65" s="30"/>
+      <c r="C65" s="45" t="s">
+        <v>49</v>
+      </c>
+      <c r="D65" s="45"/>
       <c r="E65" s="1"/>
       <c r="F65" s="1"/>
       <c r="G65" s="1"/>
@@ -3210,10 +3209,10 @@
     <row r="66" spans="1:13" ht="24.6" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A66" s="1"/>
       <c r="B66" s="16"/>
-      <c r="C66" s="30" t="s">
-        <v>51</v>
-      </c>
-      <c r="D66" s="30"/>
+      <c r="C66" s="45" t="s">
+        <v>50</v>
+      </c>
+      <c r="D66" s="45"/>
       <c r="E66" s="1"/>
       <c r="F66" s="1"/>
       <c r="G66" s="1"/>
@@ -3227,10 +3226,10 @@
     <row r="67" spans="1:13" ht="21" x14ac:dyDescent="0.35">
       <c r="A67" s="1"/>
       <c r="B67" s="16"/>
-      <c r="C67" s="30" t="s">
-        <v>52</v>
-      </c>
-      <c r="D67" s="30"/>
+      <c r="C67" s="45" t="s">
+        <v>51</v>
+      </c>
+      <c r="D67" s="45"/>
       <c r="E67" s="1"/>
       <c r="F67" s="1"/>
       <c r="G67" s="1"/>
@@ -3244,10 +3243,10 @@
     <row r="68" spans="1:13" ht="21" x14ac:dyDescent="0.35">
       <c r="A68" s="1"/>
       <c r="B68" s="16"/>
-      <c r="C68" s="21" t="s">
-        <v>53</v>
-      </c>
-      <c r="D68" s="21"/>
+      <c r="C68" s="28" t="s">
+        <v>52</v>
+      </c>
+      <c r="D68" s="28"/>
       <c r="E68" s="1"/>
       <c r="F68" s="1"/>
       <c r="G68" s="1"/>
@@ -3261,10 +3260,10 @@
     <row r="69" spans="1:13" ht="21" x14ac:dyDescent="0.35">
       <c r="A69" s="1"/>
       <c r="B69" s="16"/>
-      <c r="C69" s="21" t="s">
-        <v>54</v>
-      </c>
-      <c r="D69" s="21"/>
+      <c r="C69" s="28" t="s">
+        <v>53</v>
+      </c>
+      <c r="D69" s="28"/>
       <c r="E69" s="1"/>
       <c r="F69" s="1"/>
       <c r="G69" s="1"/>
@@ -3325,7 +3324,7 @@
     <row r="73" spans="1:13" ht="145.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A73" s="1"/>
       <c r="B73" s="25" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C73" s="25"/>
       <c r="D73" s="25"/>
@@ -3356,20 +3355,20 @@
     </row>
     <row r="75" spans="1:13" ht="25.2" x14ac:dyDescent="0.3">
       <c r="A75" s="1"/>
-      <c r="B75" s="26" t="s">
+      <c r="B75" s="42" t="s">
         <v>32</v>
       </c>
-      <c r="C75" s="27"/>
-      <c r="D75" s="27"/>
-      <c r="E75" s="27"/>
-      <c r="F75" s="27"/>
-      <c r="G75" s="27"/>
-      <c r="H75" s="27"/>
-      <c r="I75" s="27"/>
-      <c r="J75" s="27"/>
-      <c r="K75" s="27"/>
-      <c r="L75" s="27"/>
-      <c r="M75" s="27"/>
+      <c r="C75" s="43"/>
+      <c r="D75" s="43"/>
+      <c r="E75" s="43"/>
+      <c r="F75" s="43"/>
+      <c r="G75" s="43"/>
+      <c r="H75" s="43"/>
+      <c r="I75" s="43"/>
+      <c r="J75" s="43"/>
+      <c r="K75" s="43"/>
+      <c r="L75" s="43"/>
+      <c r="M75" s="43"/>
     </row>
     <row r="76" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A76" s="1"/>
@@ -3386,10 +3385,10 @@
       <c r="L76" s="1"/>
       <c r="M76" s="1"/>
     </row>
-    <row r="77" spans="1:13" ht="84" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:13" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A77" s="1"/>
       <c r="B77" s="25" t="s">
-        <v>33</v>
+        <v>70</v>
       </c>
       <c r="C77" s="25"/>
       <c r="D77" s="25"/>
@@ -3421,19 +3420,19 @@
     <row r="79" spans="1:13" ht="24.6" x14ac:dyDescent="0.3">
       <c r="A79" s="1"/>
       <c r="B79" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="C79" s="28"/>
-      <c r="D79" s="28"/>
-      <c r="E79" s="28"/>
-      <c r="F79" s="28"/>
-      <c r="G79" s="28"/>
-      <c r="H79" s="28"/>
-      <c r="I79" s="28"/>
-      <c r="J79" s="28"/>
-      <c r="K79" s="28"/>
-      <c r="L79" s="28"/>
-      <c r="M79" s="28"/>
+        <v>33</v>
+      </c>
+      <c r="C79" s="31"/>
+      <c r="D79" s="31"/>
+      <c r="E79" s="31"/>
+      <c r="F79" s="31"/>
+      <c r="G79" s="31"/>
+      <c r="H79" s="31"/>
+      <c r="I79" s="31"/>
+      <c r="J79" s="31"/>
+      <c r="K79" s="31"/>
+      <c r="L79" s="31"/>
+      <c r="M79" s="31"/>
     </row>
     <row r="80" spans="1:13" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A80" s="1"/>
@@ -3452,20 +3451,20 @@
     </row>
     <row r="81" spans="1:13" ht="71.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A81" s="1"/>
-      <c r="B81" s="22" t="s">
-        <v>55</v>
-      </c>
-      <c r="C81" s="22"/>
-      <c r="D81" s="22"/>
-      <c r="E81" s="22"/>
-      <c r="F81" s="22"/>
-      <c r="G81" s="22"/>
-      <c r="H81" s="22"/>
-      <c r="I81" s="22"/>
-      <c r="J81" s="22"/>
-      <c r="K81" s="22"/>
-      <c r="L81" s="22"/>
-      <c r="M81" s="22"/>
+      <c r="B81" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="C81" s="21"/>
+      <c r="D81" s="21"/>
+      <c r="E81" s="21"/>
+      <c r="F81" s="21"/>
+      <c r="G81" s="21"/>
+      <c r="H81" s="21"/>
+      <c r="I81" s="21"/>
+      <c r="J81" s="21"/>
+      <c r="K81" s="21"/>
+      <c r="L81" s="21"/>
+      <c r="M81" s="21"/>
     </row>
     <row r="82" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A82" s="1"/>
@@ -3544,16 +3543,22 @@
     </row>
   </sheetData>
   <mergeCells count="42">
-    <mergeCell ref="B14:M14"/>
-    <mergeCell ref="B15:M15"/>
-    <mergeCell ref="B16:M16"/>
-    <mergeCell ref="B18:M18"/>
-    <mergeCell ref="C44:D44"/>
-    <mergeCell ref="C46:D46"/>
-    <mergeCell ref="C47:D47"/>
-    <mergeCell ref="C48:D48"/>
-    <mergeCell ref="C49:D49"/>
-    <mergeCell ref="C45:D45"/>
+    <mergeCell ref="C69:D69"/>
+    <mergeCell ref="B81:M81"/>
+    <mergeCell ref="B58:M58"/>
+    <mergeCell ref="B71:M71"/>
+    <mergeCell ref="B73:M73"/>
+    <mergeCell ref="B75:M75"/>
+    <mergeCell ref="B77:M77"/>
+    <mergeCell ref="B79:M79"/>
+    <mergeCell ref="C60:D60"/>
+    <mergeCell ref="C61:D61"/>
+    <mergeCell ref="C62:D62"/>
+    <mergeCell ref="C63:D63"/>
+    <mergeCell ref="C64:D64"/>
+    <mergeCell ref="C65:D65"/>
+    <mergeCell ref="C66:D66"/>
+    <mergeCell ref="C67:D67"/>
     <mergeCell ref="C68:D68"/>
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="B2:M2"/>
@@ -3570,22 +3575,16 @@
     <mergeCell ref="B36:M36"/>
     <mergeCell ref="B38:M38"/>
     <mergeCell ref="B54:M54"/>
-    <mergeCell ref="C69:D69"/>
-    <mergeCell ref="B81:M81"/>
-    <mergeCell ref="B58:M58"/>
-    <mergeCell ref="B71:M71"/>
-    <mergeCell ref="B73:M73"/>
-    <mergeCell ref="B75:M75"/>
-    <mergeCell ref="B77:M77"/>
-    <mergeCell ref="B79:M79"/>
-    <mergeCell ref="C60:D60"/>
-    <mergeCell ref="C61:D61"/>
-    <mergeCell ref="C62:D62"/>
-    <mergeCell ref="C63:D63"/>
-    <mergeCell ref="C64:D64"/>
-    <mergeCell ref="C65:D65"/>
-    <mergeCell ref="C66:D66"/>
-    <mergeCell ref="C67:D67"/>
+    <mergeCell ref="C46:D46"/>
+    <mergeCell ref="C47:D47"/>
+    <mergeCell ref="C48:D48"/>
+    <mergeCell ref="C49:D49"/>
+    <mergeCell ref="C45:D45"/>
+    <mergeCell ref="B14:M14"/>
+    <mergeCell ref="B15:M15"/>
+    <mergeCell ref="B16:M16"/>
+    <mergeCell ref="B18:M18"/>
+    <mergeCell ref="C44:D44"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>